<commit_message>
Build provenance-aware world lubricant catalog seed
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -641,12 +641,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Public catalog; count observed 2026-07-20</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ingest official JASO filed oil registries
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -613,134 +613,146 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>JASO 4T filed oils</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global filed list</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official PDF registry</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+          <t>https://www.jalos.or.jp/onfile/pdf/4T_EV_LIST.pdf</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1246</v>
+        <v>2612</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>filed rows</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>List dated 2026-07-01; 2,611 unique oil codes</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>JASO diesel filed oils</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global filed list</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Official PDF registry</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
+          <t>https://www.jalos.or.jp/onfile/pdf/DEO_EV_LIST.pdf</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>filed rows</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>List dated 2026-07-01; 419 unique oil codes</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>JASO 2T filed oils</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global filed list</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>Official PDF registry</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
+          <t>https://www.jalos.or.jp/onfile/pdf/2T_EV_LIST.pdf</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>599</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>filed rows</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>List dated 2026-07-01; 599 unique oil codes</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1115</v>
+        <v>1246</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -749,201 +761,207 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>686</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.epc.shell.com/?lang=eng</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>active references</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1115</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>686</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -953,19 +971,19 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -977,29 +995,29 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1011,41 +1029,41 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1060,14 +1078,14 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1079,29 +1097,29 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1113,7 +1131,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1128,14 +1146,14 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1147,7 +1165,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1162,14 +1180,14 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1181,7 +1199,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1191,19 +1209,19 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1215,7 +1233,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1225,19 +1243,19 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1249,7 +1267,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1264,14 +1282,14 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1283,7 +1301,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1293,29 +1311,131 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Repsol</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>https://lubricants.repsol.com/en/products/</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H21"/>
+  <autoFilter ref="A1:H24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Gate API and NSF directories pending feed access
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,12 +555,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -733,7 +733,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -743,173 +743,161 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>1115</v>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.epc.shell.com/?lang=eng</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>686</v>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -921,149 +909,161 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>19000</v>
+        <v>1115</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>686</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1097,41 +1097,41 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1146,14 +1146,14 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1165,29 +1165,29 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1199,7 +1199,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1214,14 +1214,14 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1233,7 +1233,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1248,14 +1248,14 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1282,14 +1282,14 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1301,7 +1301,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1311,12 +1311,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
@@ -1335,7 +1335,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1345,19 +1345,19 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1369,7 +1369,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1379,19 +1379,19 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1403,7 +1403,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1413,29 +1413,97 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H24"/>
+  <autoFilter ref="A1:H26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest official licensed lubricant registries
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,15 +555,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="41" customWidth="1" min="8" max="8"/>
   </cols>
@@ -733,439 +733,469 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>NMMA TC-W3</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global licensed list</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official marine-oil registry</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
+          <t>https://www.nmma.org/certification/oil/tc-w3</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>licensed products</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>2026 registered two-stroke-cycle marine oils</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>NMMA FC-W</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global licensed list</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official marine-oil registry</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+          <t>https://www.nmma.org/certification/oil/fc-w</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>licensed products</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>2026 registered four-stroke-cycle marine oils</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NMMA FC-W(CAT)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global licensed list</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official marine-oil registry</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+          <t>https://www.nmma.org/certification/oil/fc-wcat</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1246</v>
+        <v>3</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>licensed products</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>2026 catalyst-compatible marine oils</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>GM dexos1 Gen3</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global licensed list</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Official OEM licensing registry</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+          <t>https://www.gmdexos.com/brands/dexos1_3/index.html</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1575</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Includes supplier, viscosity and GM licence number</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>GM dexos2</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global licensed list</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>Official OEM licensing registry</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+          <t>https://www.gmdexos.com/brands/dexos2/index.html</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>One source licence-number collision retained explicitly</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>GM dexosD</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global licensed list</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Official OEM licensing registry</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
+          <t>https://www.gmdexos.com/brands/dexosd/index.html</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1115</v>
+        <v>41</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>licensed product rows</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Includes supplier, viscosity and GM licence number</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>GM dexosR</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Global licensed list</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Official OEM licensing registry</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.gmdexos.com/brands/dexosr/index.html</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>686</v>
+        <v>8</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>licensed product rows</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Includes supplier, viscosity and GM licence number</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>NLGI certified products</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global licensed list</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official grease certification registry</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.nlgi.org/about-us/high-performance-multiuse-grease/</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>19000</v>
+        <v>279</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>certified product rows</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>HPM, GC-LB, GC and LB with enhancement tags</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>EU Ecolabel lubricants</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>EU/EEA</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Official open-data API</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
+          <t>https://apps.data.env.service.ec.europa.eu/dataquery/v2/ecolabel/products?group_id__eq=57&amp;limit=1000</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>certified product rows</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Public ECAT API; licence, holder, availability and expiry retained</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>USDA BioPreferred</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>United States / global suppliers</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official voluntary product catalog</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.biopreferred.gov/BioPreferred/faces/catalog/Catalog.xhtml</t>
         </is>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Lubricants, greases, hydraulic, heat-transfer, transformer and metalworking fluids; machine-readable feed still under review</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>feed_discovery</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1175,31 +1205,37 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1209,31 +1245,31 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1243,133 +1279,151 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>1115</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>686</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1379,19 +1433,19 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1403,7 +1457,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1413,19 +1467,19 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1437,41 +1491,41 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1486,24 +1540,364 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
+          <t>Specialty industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>SKF</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Maintenance and lubrication products</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Petro-Canada Lubricants</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Chevron Lubricants</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Delo, Havoline and industrial products</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Valvoline</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.valvolineglobal.com/en/products/</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Automotive oils and fluids; region-specific availability</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>PETRONAS Lubricants</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>https://global.pli-petronas.com/products</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>ENEOS</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Idemitsu</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Repsol</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>https://lubricants.repsol.com/en/products/</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H26"/>
+  <autoFilter ref="A1:H36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest USDA BioPreferred and ZF approvals
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,15 +555,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="41" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1111,57 +1111,69 @@
           <t>https://www.biopreferred.gov/BioPreferred/faces/catalog/Catalog.xhtml</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
+      <c r="E14" s="2" t="n">
+        <v>892</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>unique product IDs</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Lubricants, greases, hydraulic, heat-transfer, transformer and metalworking fluids; machine-readable feed still under review</t>
+          <t>1,387 category occurrences merged by USDA product ID; descriptions excluded from republication</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>feed_discovery</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>1498</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>unique approval numbers</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1171,31 +1183,31 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1205,71 +1217,71 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1279,59 +1291,53 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>1115</v>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1348,7 +1354,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1358,11 +1364,11 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>686</v>
+        <v>1115</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1371,7 +1377,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1383,81 +1389,87 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>19000</v>
+        <v>686</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1467,19 +1479,19 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1491,12 +1503,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1506,82 +1518,82 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1593,29 +1605,29 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1627,7 +1639,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1642,14 +1654,14 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1661,7 +1673,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1676,14 +1688,14 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1695,7 +1707,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1710,14 +1722,14 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1729,7 +1741,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1744,7 +1756,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
@@ -1763,7 +1775,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1773,12 +1785,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
@@ -1797,7 +1809,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1812,14 +1824,14 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1831,7 +1843,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1841,12 +1853,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
@@ -1865,7 +1877,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1880,24 +1892,58 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H36"/>
+  <autoFilter ref="A1:H37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest Allison approved transmission fluids
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,10 +555,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
@@ -1173,41 +1173,47 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>approved products</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1217,31 +1223,31 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1251,71 +1257,71 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1325,59 +1331,53 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="n">
-        <v>1115</v>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1404,11 +1404,11 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>686</v>
+        <v>1115</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1429,81 +1429,87 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>19000</v>
+        <v>686</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1513,19 +1519,19 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1537,12 +1543,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1552,82 +1558,82 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1639,29 +1645,29 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1673,7 +1679,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1688,14 +1694,14 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1707,7 +1713,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1722,14 +1728,14 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1741,7 +1747,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1756,14 +1762,14 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1775,7 +1781,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1790,7 +1796,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
@@ -1809,7 +1815,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1819,12 +1825,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
@@ -1843,7 +1849,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1858,14 +1864,14 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1877,7 +1883,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1887,12 +1893,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
@@ -1911,7 +1917,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1926,24 +1932,58 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest Driventic DIWA approved oils
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,10 +555,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
@@ -1213,41 +1213,47 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>approved products</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1257,31 +1263,31 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1291,71 +1297,71 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1365,59 +1371,53 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n">
-        <v>1115</v>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1444,11 +1444,11 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>686</v>
+        <v>1115</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1469,81 +1469,87 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>19000</v>
+        <v>686</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1553,19 +1559,19 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1577,12 +1583,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1592,82 +1598,82 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1679,29 +1685,29 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1713,7 +1719,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1728,14 +1734,14 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1747,7 +1753,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1762,14 +1768,14 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1781,7 +1787,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1796,14 +1802,14 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1815,7 +1821,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1830,7 +1836,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
@@ -1849,7 +1855,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1859,12 +1865,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
@@ -1883,7 +1889,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1898,14 +1904,14 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1917,7 +1923,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1927,12 +1933,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
@@ -1951,7 +1957,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1966,24 +1972,58 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H38"/>
+  <autoFilter ref="A1:H39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest Mercedes-Benz Trucks DTFR approvals
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1253,41 +1253,47 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>1892</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>unique DTFR product IDs</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1297,31 +1303,31 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1331,71 +1337,71 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1405,59 +1411,53 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>1115</v>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1484,11 +1484,11 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>686</v>
+        <v>1115</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1509,81 +1509,87 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>19000</v>
+        <v>686</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1593,19 +1599,19 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1617,12 +1623,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1632,82 +1638,82 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1719,29 +1725,29 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1753,7 +1759,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1768,14 +1774,14 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1787,7 +1793,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1802,14 +1808,14 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1821,7 +1827,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1836,14 +1842,14 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1855,7 +1861,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1870,7 +1876,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
@@ -1889,7 +1895,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1899,12 +1905,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
@@ -1923,7 +1929,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1938,14 +1944,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1957,7 +1963,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1967,12 +1973,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
@@ -1991,7 +1997,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2006,24 +2012,58 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H39"/>
+  <autoFilter ref="A1:H40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest Mercedes-Benz BeVo approvals
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -563,7 +563,7 @@
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="41" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1293,41 +1293,47 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1913</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>normalized approved products</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1337,31 +1343,31 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1371,71 +1377,71 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1445,59 +1451,53 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>1115</v>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1524,11 +1524,11 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>686</v>
+        <v>1115</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1549,81 +1549,87 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>19000</v>
+        <v>686</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1633,19 +1639,19 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1657,12 +1663,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1672,82 +1678,82 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1759,29 +1765,29 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1793,7 +1799,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1808,14 +1814,14 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1827,7 +1833,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1842,14 +1848,14 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1861,7 +1867,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1876,14 +1882,14 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1895,7 +1901,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1910,7 +1916,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
@@ -1929,7 +1935,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1939,12 +1945,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
@@ -1963,7 +1969,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1978,14 +1984,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -1997,7 +2003,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2007,12 +2013,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
@@ -2031,7 +2037,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2046,24 +2052,58 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H40"/>
+  <autoFilter ref="A1:H41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest Volvo genuine lubricants and coolants
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,11 +555,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -1333,41 +1333,47 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>specific product-grade rows</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1377,31 +1383,31 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1411,71 +1417,71 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1485,59 +1491,53 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n">
-        <v>1115</v>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1564,11 +1564,11 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>686</v>
+        <v>1115</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1589,81 +1589,87 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>19000</v>
+        <v>686</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1673,19 +1679,19 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1697,12 +1703,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1712,82 +1718,82 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1799,29 +1805,29 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1833,7 +1839,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1848,14 +1854,14 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1867,7 +1873,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1882,14 +1888,14 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1901,7 +1907,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1916,14 +1922,14 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1935,7 +1941,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1950,7 +1956,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
@@ -1969,7 +1975,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1979,12 +1985,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
@@ -2003,7 +2009,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2018,14 +2024,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2037,7 +2043,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2047,12 +2053,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
@@ -2071,7 +2077,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2086,24 +2092,58 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H41"/>
+  <autoFilter ref="A1:H42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest current MAN service product recommendations
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,11 +555,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -1373,41 +1373,47 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1417,31 +1423,31 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1451,71 +1457,71 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1525,59 +1531,53 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>1115</v>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>Search by product, specification, application and equipment builder</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>686</v>
+        <v>1115</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1629,81 +1629,87 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Product finder</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>19000</v>
+        <v>686</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>Market catalog; overlaps other FUCHS markets</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1713,19 +1719,19 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1737,12 +1743,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1752,82 +1758,82 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1839,29 +1845,29 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1873,7 +1879,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1888,14 +1894,14 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1907,7 +1913,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1922,14 +1928,14 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1941,7 +1947,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1956,14 +1962,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1975,7 +1981,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1990,7 +1996,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
@@ -2009,7 +2015,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2019,12 +2025,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
@@ -2043,7 +2049,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2058,14 +2064,14 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2077,7 +2083,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2087,12 +2093,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
@@ -2111,7 +2117,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2126,24 +2132,58 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H42"/>
+  <autoFilter ref="A1:H43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS India product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -563,9 +563,9 @@
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="41" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1608,21 +1608,21 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>1115</v>
+        <v>1007</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Broad automotive, industrial, grease and metalworking portfolio</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ingest FUCHS USA product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Product finder</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1648,21 +1648,21 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>686</v>
+        <v>623</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Market catalog; overlaps other FUCHS markets</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ingest FUCHS Germany product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1669,81 +1669,87 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>19000</v>
+        <v>1464</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1753,19 +1759,19 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1777,12 +1783,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1792,82 +1798,82 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1879,29 +1885,29 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1913,7 +1919,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1928,14 +1934,14 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1947,7 +1953,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1962,14 +1968,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1981,7 +1987,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1996,14 +2002,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2015,7 +2021,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2030,7 +2036,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
@@ -2049,7 +2055,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2059,12 +2065,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
@@ -2083,7 +2089,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2098,14 +2104,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2117,7 +2123,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2127,12 +2133,12 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
@@ -2151,7 +2157,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2166,24 +2172,58 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H43"/>
+  <autoFilter ref="A1:H44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS Poland product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1709,81 +1709,87 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>19000</v>
+        <v>690</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1793,19 +1799,19 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1817,12 +1823,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1832,82 +1838,82 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1919,29 +1925,29 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1953,7 +1959,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1968,14 +1974,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1987,7 +1993,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2002,14 +2008,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2021,7 +2027,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2036,14 +2042,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2055,7 +2061,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2070,7 +2076,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
@@ -2089,7 +2095,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2099,12 +2105,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
@@ -2123,7 +2129,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2138,14 +2144,14 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2157,7 +2163,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2167,12 +2173,12 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
@@ -2191,7 +2197,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2206,24 +2212,58 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H44"/>
+  <autoFilter ref="A1:H45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS Italy product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1749,81 +1749,87 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>19000</v>
+        <v>1007</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1833,19 +1839,19 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1857,12 +1863,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1872,82 +1878,82 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1959,29 +1965,29 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1993,7 +1999,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2008,14 +2014,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2027,7 +2033,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2042,14 +2048,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2061,7 +2067,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2076,14 +2082,14 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2095,7 +2101,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2110,7 +2116,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
@@ -2129,7 +2135,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2139,12 +2145,12 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
@@ -2163,7 +2169,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2178,14 +2184,14 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2197,7 +2203,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2207,12 +2213,12 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
@@ -2231,7 +2237,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2246,24 +2252,58 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H45"/>
+  <autoFilter ref="A1:H46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS Sweden product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1789,81 +1789,87 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>19000</v>
+        <v>675</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1873,19 +1879,19 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1897,12 +1903,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1912,82 +1918,82 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1999,29 +2005,29 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2033,7 +2039,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2048,14 +2054,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2067,7 +2073,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2082,14 +2088,14 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2101,7 +2107,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2116,14 +2122,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2135,7 +2141,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2150,7 +2156,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
@@ -2169,7 +2175,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2179,12 +2185,12 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
@@ -2203,7 +2209,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2218,14 +2224,14 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2237,7 +2243,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2247,12 +2253,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
@@ -2271,7 +2277,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2286,24 +2292,58 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H46"/>
+  <autoFilter ref="A1:H47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS Spain and compress catalog database
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -479,7 +479,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1829,81 +1829,87 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>19000</v>
+        <v>938</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1913,19 +1919,19 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1937,12 +1943,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1952,82 +1958,82 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2039,29 +2045,29 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2073,7 +2079,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2088,14 +2094,14 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2107,7 +2113,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2122,14 +2128,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2141,7 +2147,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2156,14 +2162,14 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2175,7 +2181,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2190,7 +2196,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
@@ -2209,7 +2215,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2219,12 +2225,12 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
@@ -2243,7 +2249,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2258,14 +2264,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2277,7 +2283,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2287,12 +2293,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
@@ -2311,7 +2317,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2326,24 +2332,58 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H47"/>
+  <autoFilter ref="A1:H48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS France product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1869,81 +1869,87 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>19000</v>
+        <v>705</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1953,19 +1959,19 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1977,12 +1983,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1992,82 +1998,82 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2079,29 +2085,29 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2113,7 +2119,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2128,14 +2134,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2147,7 +2153,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2162,14 +2168,14 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2181,7 +2187,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2196,14 +2202,14 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2215,7 +2221,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2230,7 +2236,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
@@ -2249,7 +2255,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2259,12 +2265,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
@@ -2283,7 +2289,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2298,14 +2304,14 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2317,7 +2323,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2327,12 +2333,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
@@ -2351,7 +2357,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2366,24 +2372,58 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H48"/>
+  <autoFilter ref="A1:H49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS Turkey product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -565,7 +565,7 @@
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="43" customWidth="1" min="8" max="8"/>
+    <col width="56" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1909,81 +1909,87 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>19000</v>
+        <v>583</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1993,19 +1999,19 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2017,12 +2023,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2032,82 +2038,82 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2119,29 +2125,29 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2153,7 +2159,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2168,14 +2174,14 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2187,7 +2193,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2202,14 +2208,14 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2221,7 +2227,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2236,14 +2242,14 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2255,7 +2261,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2270,7 +2276,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
@@ -2289,7 +2295,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2299,12 +2305,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
@@ -2323,7 +2329,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2338,14 +2344,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2357,7 +2363,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2367,12 +2373,12 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
@@ -2391,7 +2397,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2406,24 +2412,58 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H49"/>
+  <autoFilter ref="A1:H50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS Canada product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1949,81 +1949,87 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>19000</v>
+        <v>289</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2033,19 +2039,19 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2057,12 +2063,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2072,82 +2078,82 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2159,29 +2165,29 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2193,7 +2199,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2208,14 +2214,14 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2227,7 +2233,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2242,14 +2248,14 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2261,7 +2267,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2276,14 +2282,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2295,7 +2301,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2310,7 +2316,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
@@ -2329,7 +2335,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2339,12 +2345,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
@@ -2363,7 +2369,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2378,14 +2384,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2397,7 +2403,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2407,12 +2413,12 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
@@ -2431,7 +2437,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2446,24 +2452,58 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H50"/>
+  <autoFilter ref="A1:H51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS China product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -565,7 +565,7 @@
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="56" customWidth="1" min="8" max="8"/>
+    <col width="57" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1989,81 +1989,87 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>19000</v>
+        <v>278</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2073,19 +2079,19 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2097,12 +2103,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2112,82 +2118,82 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2199,29 +2205,29 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2233,7 +2239,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2248,14 +2254,14 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2267,7 +2273,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2282,14 +2288,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2301,7 +2307,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2316,14 +2322,14 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2335,7 +2341,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2350,7 +2356,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
@@ -2369,7 +2375,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2379,12 +2385,12 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
@@ -2403,7 +2409,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2418,14 +2424,14 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2437,7 +2443,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2447,12 +2453,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
@@ -2471,7 +2477,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2486,24 +2492,58 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H51"/>
+  <autoFilter ref="A1:H52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS Czech product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2029,81 +2029,87 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>19000</v>
+        <v>1146</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2113,19 +2119,19 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2137,12 +2143,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2152,82 +2158,82 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2239,29 +2245,29 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2273,7 +2279,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2288,14 +2294,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2307,7 +2313,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2322,14 +2328,14 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2341,7 +2347,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2356,14 +2362,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2375,7 +2381,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2390,7 +2396,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
@@ -2409,7 +2415,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2419,12 +2425,12 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
@@ -2443,7 +2449,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2458,14 +2464,14 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2477,7 +2483,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2487,12 +2493,12 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
@@ -2511,7 +2517,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2526,24 +2532,58 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H52"/>
+  <autoFilter ref="A1:H53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest FUCHS Mexico and South Africa catalogs
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2069,149 +2069,161 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>19000</v>
+        <v>314</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>756</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>normalized product-grade rows</t>
+        </is>
+      </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Also reports more than 400 formulations; references are not normalized products</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official product catalog</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
+          <t>https://www.liqui-moly.com/en/products.html</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Automotive oils, additives, service fluids and related products</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2221,19 +2233,19 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2245,41 +2257,41 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.dupont.com/molykote.html</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ready_for_technical_review</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2294,14 +2306,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2313,29 +2325,29 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2347,7 +2359,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2362,14 +2374,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2381,7 +2393,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2396,14 +2408,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2415,7 +2427,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2430,14 +2442,14 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2449,7 +2461,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2459,12 +2471,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
@@ -2483,7 +2495,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2493,19 +2505,19 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2517,7 +2529,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2527,19 +2539,19 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2551,7 +2563,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2561,29 +2573,97 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H53"/>
+  <autoFilter ref="A1:H55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ingest historical LIQUI MOLY product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -1577,12 +1577,12 @@
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Search by product, specification, application and equipment builder</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2194,29 +2194,35 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official product catalog</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/en/products.html</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils, additives, service fluids and related products</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2272,19 +2278,25 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/molykote.html</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Hundreds of specialty lubricants; detailed chemistry and temperature attributes</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>ready_for_technical_review</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add current LIQUI MOLY catalog lifecycle
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -563,7 +563,7 @@
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="57" customWidth="1" min="8" max="8"/>
   </cols>
@@ -2229,46 +2229,52 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2278,88 +2284,88 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Specialty industrial lubricants</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2371,29 +2377,29 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2405,7 +2411,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2420,14 +2426,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Industrial, automotive, food-grade and specialty fluids</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2439,7 +2445,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2454,14 +2460,14 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2473,7 +2479,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2488,14 +2494,14 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2507,7 +2513,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2522,7 +2528,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
@@ -2541,7 +2547,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2551,12 +2557,12 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
@@ -2575,7 +2581,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2590,14 +2596,14 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2609,7 +2615,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2619,12 +2625,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
@@ -2643,7 +2649,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2658,24 +2664,58 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H55"/>
+  <autoFilter ref="A1:H56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Brazil ANP lubricant registry
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,11 +555,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -1133,35 +1133,35 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>ANP Brazil lubricant registry</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Brazil / imported and national products</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official weekly open-government CSV</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://www.gov.br/anp/pt-br/centrais-de-conteudo/dados-abertos/registro-de-oleos-e-graxas-lubrificantes</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1498</v>
+        <v>12664</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>14,960 source rows; 8,193 registration numbers; holder, producer, use, SAE/ISO/NLGI, performance, composition and package facts retained</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1173,7 +1173,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1183,25 +1183,25 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1213,7 +1213,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1223,16 +1223,16 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1263,25 +1263,25 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1293,7 +1293,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1308,20 +1308,20 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1333,35 +1333,35 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1373,22 +1373,22 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
@@ -1396,12 +1396,12 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1413,41 +1413,47 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1457,31 +1463,31 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1491,71 +1497,71 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1565,64 +1571,58 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1644,11 +1644,11 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1684,11 +1684,11 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1764,11 +1764,11 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1804,11 +1804,11 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1937,12 +1937,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1977,12 +1977,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2017,12 +2017,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2124,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2149,80 +2149,80 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2234,81 +2234,87 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2318,122 +2324,122 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Specialty industrial lubricants</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Industrial, automotive, food-grade and specialty fluids</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2445,7 +2451,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2460,26 +2466,26 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2494,14 +2500,14 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2513,7 +2519,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2528,14 +2534,14 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2547,7 +2553,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2562,7 +2568,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
@@ -2581,7 +2587,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2591,12 +2597,12 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
@@ -2615,7 +2621,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2630,14 +2636,14 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2649,7 +2655,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2659,12 +2665,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
@@ -2683,7 +2689,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2698,24 +2704,92 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
           <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>discovery</t>
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
+  <autoFilter ref="A1:H58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Indonesia NPT lubricant registry
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,10 +555,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="41" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
@@ -1173,35 +1173,35 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>Indonesia NPT lubricant registry</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Indonesia / registered products</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official public-government registry PDF</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://migas.esdm.go.id/daftar-umum-pelumas</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1498</v>
+        <v>12626</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>published product rows</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>2021-2025 list: 12,575 rows with NPT, 51 source placeholders; expiry lifecycle is computed and labelled as an inference</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1213,7 +1213,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1223,25 +1223,25 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1263,16 +1263,16 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1293,7 +1293,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1303,25 +1303,25 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1333,7 +1333,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1348,20 +1348,20 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1373,35 +1373,35 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1413,22 +1413,22 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
@@ -1436,12 +1436,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1453,41 +1453,47 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1497,31 +1503,31 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1531,71 +1537,71 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1605,64 +1611,58 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1684,11 +1684,11 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1764,11 +1764,11 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1804,11 +1804,11 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1977,12 +1977,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2017,12 +2017,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,12 +2057,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2124,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2164,11 +2164,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2189,80 +2189,80 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2274,81 +2274,87 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2358,54 +2364,54 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2417,75 +2423,75 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2500,26 +2506,26 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2534,14 +2540,14 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2553,7 +2559,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2568,14 +2574,14 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2587,7 +2593,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2602,7 +2608,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
@@ -2621,7 +2627,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2631,12 +2637,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
@@ -2655,7 +2661,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2670,14 +2676,14 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2689,7 +2695,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2699,12 +2705,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
@@ -2723,7 +2729,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2738,14 +2744,14 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2757,39 +2763,73 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
           <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H58"/>
+  <autoFilter ref="A1:H59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add DLA qualified lubricant products
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,12 +555,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="41" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="58" customWidth="1" min="6" max="6"/>
@@ -1213,35 +1213,35 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1498</v>
+        <v>431</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1263,25 +1263,25 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1293,7 +1293,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1303,16 +1303,16 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1333,7 +1333,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1343,25 +1343,25 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1388,20 +1388,20 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1413,35 +1413,35 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1453,22 +1453,22 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1493,41 +1493,47 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1537,31 +1543,31 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1571,71 +1577,71 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1645,64 +1651,58 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1764,11 +1764,11 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1804,11 +1804,11 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2017,12 +2017,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,12 +2057,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,12 +2097,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2124,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2164,11 +2164,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2229,80 +2229,80 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2314,81 +2314,87 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2398,54 +2404,54 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2457,75 +2463,75 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2540,26 +2546,26 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2574,14 +2580,14 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2593,7 +2599,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2608,14 +2614,14 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2627,7 +2633,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2642,7 +2648,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
@@ -2661,7 +2667,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2671,12 +2677,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
@@ -2695,7 +2701,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2710,14 +2716,14 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2729,7 +2735,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2739,12 +2745,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
@@ -2763,7 +2769,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2778,14 +2784,14 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2797,39 +2803,113 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n"/>
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
           <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Detroit / Daimler Truck DFS</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>North America / global suppliers</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Official approved-fluids PDF lists</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>661</v>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>approval occurrences</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>written_permission_required</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H59"/>
+  <autoFilter ref="A1:H61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Extend DLA catalog with lubricant chemistry
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,12 +555,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="49" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="58" customWidth="1" min="6" max="6"/>
@@ -1253,47 +1253,47 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1303,25 +1303,25 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1333,7 +1333,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1343,16 +1343,16 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1383,25 +1383,25 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1428,20 +1428,20 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1453,35 +1453,35 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1493,22 +1493,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
@@ -1516,12 +1516,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1533,41 +1533,47 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1577,31 +1583,31 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1611,71 +1617,71 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1685,64 +1691,58 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1764,11 +1764,11 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1804,11 +1804,11 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,12 +2057,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,12 +2097,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2124,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,12 +2137,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2164,11 +2164,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2244,11 +2244,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2269,80 +2269,80 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2354,81 +2354,87 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2438,54 +2444,54 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2497,75 +2503,75 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2580,26 +2586,26 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2614,14 +2620,14 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2633,7 +2639,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2648,14 +2654,14 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2667,7 +2673,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2682,7 +2688,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
@@ -2701,7 +2707,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2711,12 +2717,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
@@ -2735,7 +2741,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2750,14 +2756,14 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2769,7 +2775,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2779,12 +2785,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
@@ -2803,7 +2809,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2818,14 +2824,14 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2837,79 +2843,113 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E61" s="2" t="n">
+      <c r="E62" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H61"/>
+  <autoFilter ref="A1:H62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Blue Angel certified lubricants
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1213,35 +1213,35 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Blue Angel DE-UZ 178</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Germany / certified products</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product registry with XLSX export</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.blauer-engel.de/de/produktwelt/schmierstoffe-und-hydraulikfluessigkeiten</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>431</v>
+        <v>148</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>normalized certified products</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>149 export rows and product cards; one exact duplicate identity merged; 159 category occurrences across seven official lubricant categories; contact and marketing fields excluded</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1281,59 +1281,59 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1343,25 +1343,25 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1383,16 +1383,16 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1423,25 +1423,25 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1468,20 +1468,20 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1493,35 +1493,35 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1533,22 +1533,22 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -1556,12 +1556,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1573,41 +1573,47 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1617,31 +1623,31 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1651,71 +1657,71 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1725,64 +1731,58 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1804,11 +1804,11 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,12 +2097,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2124,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,12 +2137,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2164,11 +2164,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2177,12 +2177,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2244,11 +2244,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2284,11 +2284,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2309,80 +2309,80 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2394,81 +2394,87 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2478,54 +2484,54 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2537,75 +2543,75 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2620,26 +2626,26 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2654,14 +2660,14 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2673,7 +2679,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2688,14 +2694,14 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2707,7 +2713,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2722,7 +2728,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
@@ -2741,7 +2747,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2751,12 +2757,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
@@ -2775,7 +2781,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2790,14 +2796,14 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2809,7 +2815,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2819,12 +2825,12 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
@@ -2843,7 +2849,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2858,14 +2864,14 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2877,79 +2883,113 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="E63" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H62"/>
+  <autoFilter ref="A1:H63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Korea ecolabel lubricant registry
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1253,35 +1253,35 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Korea Eco-Label EL611</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Republic of Korea / certified products</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official open-government ecolabel CSV</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.data.go.kr/data/15043624/fileData.do</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>431</v>
+        <v>20</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>normalized certified products</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>240,695 file rows observed versus 99,602 in portal metadata; exact EL611 filter yields 21 lubricant rows and 20 product identities; unrestricted use; business and location identifiers excluded</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1293,75 +1293,75 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>25</v>
+        <v>124</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1498</v>
+        <v>431</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1373,47 +1373,47 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1423,25 +1423,25 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>226</v>
+        <v>1498</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1463,25 +1463,25 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>1892</v>
+        <v>104</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1493,7 +1493,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1503,25 +1503,25 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>1913</v>
+        <v>226</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1533,35 +1533,35 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>32</v>
+        <v>1892</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1573,35 +1573,35 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1613,75 +1613,87 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>specific product-grade rows</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1691,178 +1703,166 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.epc.shell.com/?lang=eng</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>623</v>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1464</v>
+        <v>1007</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>690</v>
+        <v>623</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1007</v>
+        <v>1464</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>938</v>
+        <v>1007</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>705</v>
+        <v>675</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2124,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>583</v>
+        <v>938</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,12 +2137,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2164,11 +2164,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>289</v>
+        <v>705</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>278</v>
+        <v>583</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2217,12 +2217,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2244,11 +2244,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>1146</v>
+        <v>289</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2257,12 +2257,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2284,11 +2284,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>314</v>
+        <v>278</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>756</v>
+        <v>1146</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2349,201 +2349,207 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>19000</v>
+        <v>314</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>419</v>
+        <v>756</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>447</v>
+        <v>19000</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>170</v>
+        <v>447</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>normalized lubricant and technical-fluid master products</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2553,65 +2559,71 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2626,14 +2638,14 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2645,29 +2657,29 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2679,7 +2691,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2694,26 +2706,26 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2728,14 +2740,14 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2747,7 +2759,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2762,14 +2774,14 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2781,7 +2793,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2791,12 +2803,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
@@ -2815,7 +2827,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2825,19 +2837,19 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2849,7 +2861,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2859,19 +2871,19 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2883,7 +2895,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2893,19 +2905,19 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2917,79 +2929,147 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E63" s="2" t="n">
+      <c r="E65" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H63"/>
+  <autoFilter ref="A1:H65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Korea ecolabel washer fluids
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1293,87 +1293,87 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>Korea Eco-Label EL509</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>Republic of Korea / certified products</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official open-government ecolabel CSV</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://www.data.go.kr/data/15043624/fileData.do</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>124</v>
+        <v>9</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>normalized certified technical fluids</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>Exact EL509 filter yields 11 vehicle glass washer fluid rows and nine product identities after package-model merging; unrestricted use; business and location identifiers excluded</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1392,7 +1392,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1401,59 +1401,59 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1463,25 +1463,25 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1493,7 +1493,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1503,16 +1503,16 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1533,7 +1533,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1543,25 +1543,25 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1573,7 +1573,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1588,20 +1588,20 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1613,35 +1613,35 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,22 +1653,22 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
@@ -1676,12 +1676,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1693,41 +1693,47 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1737,31 +1743,31 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1771,71 +1777,71 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1845,64 +1851,58 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2124,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2164,11 +2164,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2217,12 +2217,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2244,11 +2244,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2257,12 +2257,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2284,11 +2284,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2297,12 +2297,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2364,11 +2364,11 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2404,11 +2404,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2429,80 +2429,80 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2514,81 +2514,87 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2598,54 +2604,54 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2657,75 +2663,75 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2740,26 +2746,26 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2774,14 +2780,14 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2793,7 +2799,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2808,14 +2814,14 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2827,7 +2833,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2842,7 +2848,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
@@ -2861,7 +2867,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2871,12 +2877,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
@@ -2895,7 +2901,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2910,14 +2916,14 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2929,7 +2935,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2939,12 +2945,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
@@ -2963,7 +2969,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -2978,14 +2984,14 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E63" s="2" t="n"/>
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -2997,79 +3003,113 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E65" s="2" t="n">
+      <c r="E66" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H65"/>
+  <autoFilter ref="A1:H66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add UAE product conformity lubricants
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,11 +555,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -1333,87 +1333,87 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>UAE MOIAT Product Conformity</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>United Arab Emirates / international certified products</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official open-government certification registry</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://moiat.gov.ae/en/open-data/product-conformity-data</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>124</v>
+        <v>1840</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>normalized product/model identities</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>131 listing pages; 1,236 certificates; 3,176 product-certificate occurrences; explicit package suffixes and certificate renewals merged; 111 products active at snapshot; open-data page permits unrestricted reuse</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1441,59 +1441,59 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1503,25 +1503,25 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1533,7 +1533,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1543,16 +1543,16 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1573,7 +1573,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1583,25 +1583,25 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1628,20 +1628,20 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,35 +1653,35 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1693,22 +1693,22 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
@@ -1716,12 +1716,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1733,41 +1733,47 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1777,31 +1783,31 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>feed_or_access_request_required</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1811,71 +1817,71 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1885,64 +1891,58 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2124,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2164,11 +2164,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2244,11 +2244,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2257,12 +2257,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2284,11 +2284,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2297,12 +2297,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2337,12 +2337,12 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2364,11 +2364,11 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2404,11 +2404,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2469,80 +2469,80 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2554,81 +2554,87 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2638,54 +2644,54 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2697,75 +2703,75 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2780,26 +2786,26 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2814,14 +2820,14 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2833,7 +2839,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2848,14 +2854,14 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2867,7 +2873,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2882,7 +2888,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
@@ -2901,7 +2907,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2911,12 +2917,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
@@ -2935,7 +2941,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2950,14 +2956,14 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -2969,7 +2975,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -2979,12 +2985,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n"/>
@@ -3003,7 +3009,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3018,14 +3024,14 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3037,79 +3043,113 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n"/>
+      <c r="F66" s="2" t="n"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E66" s="2" t="n">
+      <c r="E67" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H66"/>
+  <autoFilter ref="A1:H67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add EPA lubricant products and registry counts
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,10 +555,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
     <col width="57" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
@@ -1093,75 +1093,75 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>USDA BioPreferred</t>
+          <t>Nordic Swan / EU Ecolabel cross-check</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>United States / global suppliers</t>
+          <t>Nordic product search</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Official voluntary product catalog</t>
+          <t>Official CSV export</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>https://www.biopreferred.gov/BioPreferred/faces/catalog/Catalog.xhtml</t>
+          <t>https://www.svanen.se/en/product-types/lubricating-grease/?format=Csv</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>892</v>
+        <v>60</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>unique product IDs</t>
+          <t>exported product rows</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>1,387 category occurrences merged by USDA product ID; descriptions excluded from republication</t>
+          <t>All 60 are EU Ecolabel / EU27 Lubricants and reconcile to existing ECAT licences; retained as secondary evidence without duplicate canonical rows</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>crosschecked_no_new_canonical_rows</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ANP Brazil lubricant registry</t>
+          <t>USDA BioPreferred</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Brazil / imported and national products</t>
+          <t>United States / global suppliers</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Official weekly open-government CSV</t>
+          <t>Official voluntary product catalog</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.br/anp/pt-br/centrais-de-conteudo/dados-abertos/registro-de-oleos-e-graxas-lubrificantes</t>
+          <t>https://www.biopreferred.gov/BioPreferred/faces/catalog/Catalog.xhtml</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>12664</v>
+        <v>892</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows</t>
+          <t>unique product IDs</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>14,960 source rows; 8,193 registration numbers; holder, producer, use, SAE/ISO/NLGI, performance, composition and package facts retained</t>
+          <t>1,387 category occurrences merged by USDA product ID; descriptions excluded from republication</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1173,35 +1173,35 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Indonesia NPT lubricant registry</t>
+          <t>ANP Brazil lubricant registry</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Indonesia / registered products</t>
+          <t>Brazil / imported and national products</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Official public-government registry PDF</t>
+          <t>Official weekly open-government CSV</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>https://migas.esdm.go.id/daftar-umum-pelumas</t>
+          <t>https://www.gov.br/anp/pt-br/centrais-de-conteudo/dados-abertos/registro-de-oleos-e-graxas-lubrificantes</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>12626</v>
+        <v>12664</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>published product rows</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2021-2025 list: 12,575 rows with NPT, 51 source placeholders; expiry lifecycle is computed and labelled as an inference</t>
+          <t>14,960 source rows; 8,193 registration numbers; holder, producer, use, SAE/ISO/NLGI, performance, composition and package facts retained</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1213,35 +1213,35 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Blue Angel DE-UZ 178</t>
+          <t>Indonesia NPT lubricant registry</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Germany / certified products</t>
+          <t>Indonesia / registered products</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product registry with XLSX export</t>
+          <t>Official public-government registry PDF</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://www.blauer-engel.de/de/produktwelt/schmierstoffe-und-hydraulikfluessigkeiten</t>
+          <t>https://migas.esdm.go.id/daftar-umum-pelumas</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>148</v>
+        <v>12626</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>normalized certified products</t>
+          <t>published product rows</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>149 export rows and product cards; one exact duplicate identity merged; 159 category occurrences across seven official lubricant categories; contact and marketing fields excluded</t>
+          <t>2021-2025 list: 12,575 rows with NPT, 51 source placeholders; expiry lifecycle is computed and labelled as an inference</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1253,26 +1253,26 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Korea Eco-Label EL611</t>
+          <t>Blue Angel DE-UZ 178</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Republic of Korea / certified products</t>
+          <t>Germany / certified products</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official open-government ecolabel CSV</t>
+          <t>Official ecolabel product registry with XLSX export</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://www.data.go.kr/data/15043624/fileData.do</t>
+          <t>https://www.blauer-engel.de/de/produktwelt/schmierstoffe-und-hydraulikfluessigkeiten</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>240,695 file rows observed versus 99,602 in portal metadata; exact EL611 filter yields 21 lubricant rows and 20 product identities; unrestricted use; business and location identifiers excluded</t>
+          <t>149 export rows and product cards; one exact duplicate identity merged; 159 category occurrences across seven official lubricant categories; contact and marketing fields excluded</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1293,7 +1293,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Korea Eco-Label EL509</t>
+          <t>Korea Eco-Label EL611</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1312,16 +1312,16 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>normalized certified technical fluids</t>
+          <t>normalized certified products</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Exact EL509 filter yields 11 vehicle glass washer fluid rows and nine product identities after package-model merging; unrestricted use; business and location identifiers excluded</t>
+          <t>240,695 file rows observed versus 99,602 in portal metadata; exact EL611 filter yields 21 lubricant rows and 20 product identities; unrestricted use; business and location identifiers excluded</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1333,35 +1333,35 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>UAE MOIAT Product Conformity</t>
+          <t>Korea Eco-Label EL509</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates / international certified products</t>
+          <t>Republic of Korea / certified products</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Official open-government certification registry</t>
+          <t>Official open-government ecolabel CSV</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>https://moiat.gov.ae/en/open-data/product-conformity-data</t>
+          <t>https://www.data.go.kr/data/15043624/fileData.do</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1840</v>
+        <v>9</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>normalized product/model identities</t>
+          <t>normalized certified technical fluids</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>131 listing pages; 1,236 certificates; 3,176 product-certificate occurrences; explicit package suffixes and certificate renewals merged; 111 products active at snapshot; open-data page permits unrestricted reuse</t>
+          <t>Exact EL509 filter yields 11 vehicle glass washer fluid rows and nine product identities after package-model merging; unrestricted use; business and location identifiers excluded</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1373,155 +1373,155 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>UAE MOIAT Product Conformity</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>United Arab Emirates / international certified products</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official open-government certification registry</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://moiat.gov.ae/en/open-data/product-conformity-data</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>124</v>
+        <v>1840</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>normalized product/model identities</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>131 listing pages; 1,236 certificates; 3,176 product-certificate occurrences; explicit package suffixes and certificate renewals merged; 111 products active at snapshot; open-data page permits unrestricted reuse</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>US EPA Safer Choice</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official open-government bulk CSV/API</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://data.epa.gov/efservice/t_safer_choice_and_design_for_the_environment/CSV</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>431</v>
+        <v>2</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>normalized explicitly named lubricant products</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>12 UPC/GTIN/MPN occurrences in 4,786 source rows merged to two medical-instrument lubricants; degreasers and grease-trap cleaners excluded</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>25</v>
+        <v>124</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>1498</v>
+        <v>431</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1533,47 +1533,47 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1583,25 +1583,25 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>226</v>
+        <v>1498</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1623,25 +1623,25 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>1892</v>
+        <v>104</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,7 +1653,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1663,25 +1663,25 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>1913</v>
+        <v>226</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1693,35 +1693,35 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>32</v>
+        <v>1892</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1733,35 +1733,35 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1773,75 +1773,87 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.api.org/products-and-services/engine-oil/eolcs-licensee-directory</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>specific product-grade rows</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>API describes the directory as free and covering active licensees/products; directory endpoint currently redirects to account sign-in</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>feed_or_access_request_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1851,178 +1863,172 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1246</v>
+        <v>35174</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>licensed product rows</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.epc.shell.com/?lang=eng</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n">
-        <v>623</v>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2040,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2044,11 +2050,11 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1464</v>
+        <v>1007</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2057,7 +2063,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2074,7 +2080,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2084,11 +2090,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>690</v>
+        <v>623</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2097,7 +2103,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2114,7 +2120,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2124,11 +2130,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1007</v>
+        <v>1464</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2137,7 +2143,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2154,7 +2160,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2164,11 +2170,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2177,7 +2183,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2194,7 +2200,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2204,11 +2210,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>938</v>
+        <v>1007</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2223,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2234,7 +2240,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2244,11 +2250,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>705</v>
+        <v>675</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2257,7 +2263,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2274,7 +2280,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2284,11 +2290,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>583</v>
+        <v>938</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2297,12 +2303,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2320,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2324,11 +2330,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>289</v>
+        <v>705</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2337,7 +2343,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2354,7 +2360,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2364,11 +2370,11 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>278</v>
+        <v>583</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2377,12 +2383,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2400,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2404,11 +2410,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>1146</v>
+        <v>289</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2417,12 +2423,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2440,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2444,11 +2450,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>314</v>
+        <v>278</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2457,7 +2463,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2474,7 +2480,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2484,11 +2490,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>756</v>
+        <v>1146</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2497,7 +2503,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2509,201 +2515,207 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>19000</v>
+        <v>314</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>419</v>
+        <v>756</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>447</v>
+        <v>19000</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>170</v>
+        <v>447</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>normalized lubricant and technical-fluid master products</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2713,65 +2725,71 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2786,14 +2804,14 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2805,29 +2823,29 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2839,7 +2857,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2854,26 +2872,26 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2888,14 +2906,14 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2907,7 +2925,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2922,14 +2940,14 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2941,7 +2959,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2951,12 +2969,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
@@ -2975,7 +2993,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -2985,19 +3003,19 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n"/>
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3009,7 +3027,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3019,19 +3037,19 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3043,7 +3061,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3053,19 +3071,19 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3077,79 +3095,147 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E66" s="2" t="n"/>
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E67" s="2" t="n">
+      <c r="E69" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H67"/>
+  <autoFilter ref="A1:H69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add KEBS S-Mark lubricant products
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -1453,87 +1453,87 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>KEBS S-Mark</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>Kenya / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://www.kebs.org/products-with-smarks/</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>124</v>
+        <v>750</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>normalized lubricant and technical-fluid products</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1561,59 +1561,59 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1623,25 +1623,25 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,7 +1653,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1663,16 +1663,16 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1693,7 +1693,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1703,25 +1703,25 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1733,7 +1733,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1748,20 +1748,20 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1773,35 +1773,35 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1813,22 +1813,22 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
@@ -1836,12 +1836,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1853,47 +1853,47 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1903,31 +1903,37 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1937,71 +1943,71 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2011,64 +2017,58 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2090,11 +2090,11 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2130,11 +2130,11 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2170,11 +2170,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2210,11 +2210,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2250,11 +2250,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2290,11 +2290,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2330,11 +2330,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2370,11 +2370,11 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2383,12 +2383,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2410,11 +2410,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2423,12 +2423,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2450,11 +2450,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2463,12 +2463,12 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2490,11 +2490,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2503,7 +2503,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2530,11 +2530,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2570,11 +2570,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2595,80 +2595,80 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2680,81 +2680,87 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2764,54 +2770,54 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2823,75 +2829,75 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2906,26 +2912,26 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2940,14 +2946,14 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2959,7 +2965,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2974,14 +2980,14 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -2993,7 +2999,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3008,7 +3014,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E63" s="2" t="n"/>
@@ -3027,7 +3033,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3037,12 +3043,12 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
@@ -3061,7 +3067,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3076,14 +3082,14 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3095,7 +3101,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3105,12 +3111,12 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E66" s="2" t="n"/>
@@ -3129,7 +3135,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3144,14 +3150,14 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3163,79 +3169,113 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E69" s="2" t="n">
+      <c r="E70" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H69"/>
+  <autoFilter ref="A1:H70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add UNBS and TBS certified lubricant products
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -1493,155 +1493,155 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>UNBS certified products</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>Uganda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://cims.unbs.go.ug/api/website/</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>124</v>
+        <v>46</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>normalized lubricant and brake-fluid products</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>TBS certified companies</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Tanzania / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.tbs.go.tz/index.php/companies</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>431</v>
+        <v>183</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>normalized lubricant, coolant and brake-fluid products</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>25</v>
+        <v>124</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>1498</v>
+        <v>431</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,47 +1653,47 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1703,25 +1703,25 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>226</v>
+        <v>1498</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1733,7 +1733,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1743,25 +1743,25 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>1892</v>
+        <v>104</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1773,7 +1773,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1783,25 +1783,25 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>1913</v>
+        <v>226</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1813,35 +1813,35 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>32</v>
+        <v>1892</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1853,35 +1853,35 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1893,81 +1893,87 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>named products</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1977,178 +1983,172 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1246</v>
+        <v>35174</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>licensed product rows</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.epc.shell.com/?lang=eng</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="n">
-        <v>623</v>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2170,11 +2170,11 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1464</v>
+        <v>1007</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2210,11 +2210,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>690</v>
+        <v>623</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2250,11 +2250,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>1007</v>
+        <v>1464</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2290,11 +2290,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2330,11 +2330,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>938</v>
+        <v>1007</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2370,11 +2370,11 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>705</v>
+        <v>675</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2410,11 +2410,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>583</v>
+        <v>938</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2423,12 +2423,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2450,11 +2450,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>289</v>
+        <v>705</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2490,11 +2490,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>278</v>
+        <v>583</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2503,12 +2503,12 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2530,11 +2530,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>1146</v>
+        <v>289</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2543,12 +2543,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2570,11 +2570,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>314</v>
+        <v>278</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2610,11 +2610,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>756</v>
+        <v>1146</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2635,201 +2635,207 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>19000</v>
+        <v>314</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>419</v>
+        <v>756</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>447</v>
+        <v>19000</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>170</v>
+        <v>447</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>normalized lubricant and technical-fluid master products</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2839,65 +2845,71 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2912,14 +2924,14 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2931,29 +2943,29 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2965,7 +2977,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2980,26 +2992,26 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3014,14 +3026,14 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E63" s="2" t="n"/>
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3033,7 +3045,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3048,14 +3060,14 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3067,7 +3079,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3077,12 +3089,12 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E65" s="2" t="n"/>
@@ -3101,7 +3113,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3111,19 +3123,19 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E66" s="2" t="n"/>
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3135,7 +3147,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3145,19 +3157,19 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3169,7 +3181,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3179,19 +3191,19 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3203,79 +3215,147 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E69" s="2" t="n"/>
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E70" s="2" t="n">
+      <c r="E72" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H70"/>
+  <autoFilter ref="A1:H72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Nigeria SON certified lubricant products
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -563,7 +563,7 @@
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="58" customWidth="1" min="6" max="6"/>
+    <col width="68" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="57" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1573,87 +1573,87 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>SON MANCAP Chemical Sector</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>Nigeria / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official mandatory product-certification PDF</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>124</v>
+        <v>608</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1672,7 +1672,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1681,59 +1681,59 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1743,25 +1743,25 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1773,7 +1773,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1783,16 +1783,16 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1813,7 +1813,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1823,25 +1823,25 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1853,7 +1853,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1868,20 +1868,20 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1893,35 +1893,35 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1933,22 +1933,22 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1973,47 +1973,47 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2023,31 +2023,37 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2057,71 +2063,71 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2131,64 +2137,58 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2210,11 +2210,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2250,11 +2250,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2290,11 +2290,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2330,11 +2330,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2370,11 +2370,11 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2410,11 +2410,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2450,11 +2450,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2490,11 +2490,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2503,12 +2503,12 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2530,11 +2530,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2543,12 +2543,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2570,11 +2570,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2583,12 +2583,12 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2610,11 +2610,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2650,11 +2650,11 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2690,11 +2690,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2703,7 +2703,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2715,80 +2715,80 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>19000</v>
+        <v>756</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -2800,81 +2800,87 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2884,54 +2890,54 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2943,75 +2949,75 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3026,26 +3032,26 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E63" s="2" t="n"/>
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3060,14 +3066,14 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3079,7 +3085,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3094,14 +3100,14 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3113,7 +3119,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3128,7 +3134,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E66" s="2" t="n"/>
@@ -3147,7 +3153,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3157,12 +3163,12 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n"/>
@@ -3181,7 +3187,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3196,14 +3202,14 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3215,7 +3221,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3225,12 +3231,12 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n"/>
@@ -3249,7 +3255,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3264,14 +3270,14 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -3283,79 +3289,113 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n"/>
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E72" s="2" t="n">
+      <c r="E73" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G72" s="2" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H72"/>
+  <autoFilter ref="A1:H73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Rwanda RSB certified lubricant products
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -1613,195 +1613,189 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>RSB S-Mark</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>Rwanda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>124</v>
+        <v>9</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>normalized currently valid lubricant products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>BIS product-certification licences</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>India / certified manufacturers</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official interactive government certification directory</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>431</v>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>normalized qualified products</t>
-        </is>
-      </c>
+          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>official_feed_or_written_access_required</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>BPCL MAK Lubricants</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>India / international markets</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>25</v>
+        <v>400</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>publicly stated minimum grades</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>1498</v>
+        <v>124</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>104</v>
+        <v>431</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1813,47 +1807,47 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>226</v>
+        <v>25</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1863,25 +1857,25 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1892</v>
+        <v>1498</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1893,7 +1887,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1903,25 +1897,25 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1913</v>
+        <v>104</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1933,35 +1927,35 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>32</v>
+        <v>226</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1973,35 +1967,35 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>32</v>
+        <v>1892</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2013,302 +2007,302 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>35174</v>
+        <v>1913</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>specific product-grade rows</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1246</v>
+        <v>32</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1007</v>
+        <v>1246</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows</t>
+          <t>products</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n">
-        <v>623</v>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.epc.shell.com/?lang=eng</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n">
-        <v>1464</v>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2314,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2330,11 +2324,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>690</v>
+        <v>1007</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2343,7 +2337,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2360,7 +2354,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2370,11 +2364,11 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>1007</v>
+        <v>623</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2383,7 +2377,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2400,7 +2394,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2410,11 +2404,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>675</v>
+        <v>1464</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2423,7 +2417,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2440,7 +2434,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2450,11 +2444,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>938</v>
+        <v>690</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2463,7 +2457,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2480,7 +2474,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2490,11 +2484,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>705</v>
+        <v>1007</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2503,7 +2497,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2520,7 +2514,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2530,11 +2524,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>583</v>
+        <v>675</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2543,12 +2537,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2554,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2570,11 +2564,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>289</v>
+        <v>938</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2583,7 +2577,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2600,7 +2594,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2610,11 +2604,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>278</v>
+        <v>705</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2623,12 +2617,12 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2634,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2650,11 +2644,11 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>1146</v>
+        <v>583</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2663,12 +2657,12 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2674,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2690,11 +2684,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>314</v>
+        <v>289</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2703,12 +2697,12 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2714,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2730,11 +2724,11 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>756</v>
+        <v>278</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2743,7 +2737,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2755,257 +2749,269 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>19000</v>
+        <v>1146</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>419</v>
+        <v>314</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>447</v>
+        <v>756</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>170</v>
+        <v>419</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3017,29 +3023,35 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="n"/>
-      <c r="F63" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3051,7 +3063,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3066,48 +3078,48 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3119,7 +3131,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3134,26 +3146,26 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E66" s="2" t="n"/>
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3168,14 +3180,14 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3187,7 +3199,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3197,19 +3209,19 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3221,7 +3233,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3231,19 +3243,19 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E69" s="2" t="n"/>
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3255,7 +3267,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3270,14 +3282,14 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -3289,7 +3301,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3299,19 +3311,19 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n"/>
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -3323,79 +3335,181 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E72" s="2" t="n"/>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="n"/>
+      <c r="F74" s="2" t="n"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="n"/>
+      <c r="F75" s="2" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E73" s="2" t="n">
+      <c r="E76" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G73" s="2" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H73"/>
+  <autoFilter ref="A1:H76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add FUCHS Brazil product catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -2869,235 +2869,235 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>19000</v>
+        <v>182</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>419</v>
+        <v>591</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.zabs.org.zm/certification</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>447</v>
+        <v>85</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>product-certification holder records</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="2" t="n"/>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>certification records</t>
+        </is>
+      </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3107,99 +3107,117 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3209,19 +3227,19 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3233,41 +3251,47 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="n"/>
-      <c r="F69" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3282,48 +3306,48 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E71" s="2" t="n"/>
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -3335,7 +3359,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3345,31 +3369,31 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E72" s="2" t="n"/>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3384,14 +3408,14 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E73" s="2" t="n"/>
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3403,7 +3427,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3418,14 +3442,14 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E74" s="2" t="n"/>
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3437,79 +3461,283 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E75" s="2" t="n"/>
       <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
+          <t>ENEOS</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Idemitsu</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="n"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Repsol</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>https://lubricants.repsol.com/en/products/</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="n"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="2" t="n"/>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="2" t="n"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="n"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E76" s="2" t="n">
+      <c r="E82" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H82" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H76"/>
+  <autoFilter ref="A1:H82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add FUCHS Norway and Hungary catalogs
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -2914,7 +2914,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2924,134 +2924,140 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>591</v>
+        <v>649</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>85</v>
+        <v>506</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>120</v>
+        <v>591</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="n"/>
-      <c r="F63" s="2" t="n"/>
+          <t>https://www.zabs.org.zm/certification</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>product-certification holder records</t>
+        </is>
+      </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3063,235 +3069,235 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="n"/>
-      <c r="F64" s="2" t="n"/>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>certification records</t>
+        </is>
+      </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>active references</t>
-        </is>
-      </c>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="n">
-        <v>419</v>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>normalized product rows</t>
-        </is>
-      </c>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n"/>
+      <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>447</v>
+        <v>19000</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="n"/>
-      <c r="F68" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>170</v>
+        <v>447</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>normalized lubricant and technical-fluid master products</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3301,65 +3307,71 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="n"/>
-      <c r="F71" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3374,14 +3386,14 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E72" s="2" t="n"/>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3393,29 +3405,29 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E73" s="2" t="n"/>
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3427,7 +3439,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3442,26 +3454,26 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E74" s="2" t="n"/>
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3476,14 +3488,14 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E75" s="2" t="n"/>
       <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -3495,7 +3507,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3510,14 +3522,14 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E76" s="2" t="n"/>
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3529,7 +3541,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -3539,12 +3551,12 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E77" s="2" t="n"/>
@@ -3563,7 +3575,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3573,19 +3585,19 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E78" s="2" t="n"/>
       <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -3597,7 +3609,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -3607,19 +3619,19 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E79" s="2" t="n"/>
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -3631,7 +3643,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3641,19 +3653,19 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E80" s="2" t="n"/>
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -3665,79 +3677,147 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E82" s="2" t="n">
+      <c r="E84" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F82" s="2" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G82" s="2" t="inlineStr">
+      <c r="G84" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H82" s="2" t="inlineStr">
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H82"/>
+  <autoFilter ref="A1:H84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add six FUCHS European product catalogs
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3004,544 +3004,580 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>591</v>
+        <v>640</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>641 embedded rows; one series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>85</v>
+        <v>599</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>120</v>
+        <v>484</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="n"/>
+          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>normalized product-grade rows</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
+          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>952</v>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>normalized product-grade rows</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>19000</v>
+        <v>966</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>419</v>
+        <v>1464</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Catalog nearly mirrors Germany but local taxonomy produces 234 fallback classifications; deferred until explicit cross-market taxonomy reconciliation</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>reviewed_taxonomy_reconciliation_required</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>447</v>
+        <v>591</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="n"/>
-      <c r="F70" s="2" t="n"/>
+          <t>https://www.zabs.org.zm/certification</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>product-certification holder records</t>
+        </is>
+      </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>170</v>
+        <v>120</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>certification records</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
         </is>
       </c>
       <c r="E72" s="2" t="n"/>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
         </is>
       </c>
       <c r="E73" s="2" t="n"/>
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="n"/>
-      <c r="F74" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="n"/>
-      <c r="F75" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="n"/>
-      <c r="F76" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -3551,19 +3587,19 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E77" s="2" t="n"/>
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -3575,41 +3611,47 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="n"/>
-      <c r="F78" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -3619,53 +3661,53 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E79" s="2" t="n"/>
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E80" s="2" t="n"/>
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -3677,7 +3719,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -3692,26 +3734,26 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3726,14 +3768,14 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E82" s="2" t="n"/>
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -3745,79 +3787,317 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E83" s="2" t="n"/>
       <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
+          <t>PETRONAS Lubricants</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>https://global.pli-petronas.com/products</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="n"/>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>ENEOS</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Idemitsu</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="n"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Repsol</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>https://lubricants.repsol.com/en/products/</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="n"/>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="n"/>
+      <c r="F89" s="2" t="n"/>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B84" s="2" t="inlineStr">
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E84" s="2" t="n">
+      <c r="E91" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr">
+      <c r="G91" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H84" s="2" t="inlineStr">
+      <c r="H91" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H84"/>
+  <autoFilter ref="A1:H91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Reconcile and add FUCHS Switzerland catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -3239,7 +3239,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3252,17 +3252,17 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Catalog nearly mirrors Germany but local taxonomy produces 234 fallback classifications; deferred until explicit cross-market taxonomy reconciliation</t>
+          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>reviewed_taxonomy_reconciliation_required</t>
+          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add eight FUCHS global market catalogs
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -3274,7 +3274,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Republic of Korea</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -3284,578 +3284,620 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>591</v>
+        <v>221</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>85</v>
+        <v>965</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>120</v>
+        <v>5</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="n"/>
-      <c r="F72" s="2" t="n"/>
+          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>496</v>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>normalized product-grade rows</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="n"/>
-      <c r="F73" s="2" t="n"/>
+          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>842</v>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>normalized product-grade rows</t>
+        </is>
+      </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>19000</v>
+        <v>966</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>419</v>
+        <v>1</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>normalized product-grade row</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>One embedded concrete product card; informational factual fields only</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>447</v>
+        <v>975</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="n"/>
-      <c r="F77" s="2" t="n"/>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>591</v>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>normalized product-grade rows observed</t>
+        </is>
+      </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://www.zabs.org.zm/certification</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>170</v>
+        <v>85</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>product-certification holder records</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="n"/>
-      <c r="F79" s="2" t="n"/>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>certification records</t>
+        </is>
+      </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
         </is>
       </c>
       <c r="E80" s="2" t="n"/>
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
         </is>
       </c>
       <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="n"/>
-      <c r="F82" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="n"/>
-      <c r="F83" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="n"/>
-      <c r="F84" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -3865,19 +3907,19 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E85" s="2" t="n"/>
       <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -3889,41 +3931,47 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="n"/>
-      <c r="F86" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -3933,53 +3981,53 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E87" s="2" t="n"/>
       <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E88" s="2" t="n"/>
       <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -3991,7 +4039,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4006,98 +4054,370 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E89" s="2" t="n"/>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E90" s="2" t="n"/>
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
+          <t>Valvoline</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.valvolineglobal.com/en/products/</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="2" t="n"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Automotive oils and fluids; region-specific availability</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>PETRONAS Lubricants</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>https://global.pli-petronas.com/products</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="n"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>ENEOS</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="n"/>
+      <c r="F93" s="2" t="n"/>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Idemitsu</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="n"/>
+      <c r="F94" s="2" t="n"/>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Repsol</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>https://lubricants.repsol.com/en/products/</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="n"/>
+      <c r="F95" s="2" t="n"/>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="n"/>
+      <c r="F96" s="2" t="n"/>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="n"/>
+      <c r="F97" s="2" t="n"/>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="n"/>
+      <c r="F98" s="2" t="n"/>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B91" s="2" t="inlineStr">
+      <c r="B99" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E91" s="2" t="n">
+      <c r="E99" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F91" s="2" t="inlineStr">
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G91" s="2" t="inlineStr">
+      <c r="G99" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H91" s="2" t="inlineStr">
+      <c r="H99" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H91"/>
+  <autoFilter ref="A1:H99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Thailand DOEB lubricant registry
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -1213,75 +1213,75 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Indonesia NPT lubricant registry</t>
+          <t>Thailand DOEB lubricant registry</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Indonesia / registered products</t>
+          <t>Thailand / registered motor oils</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Official public-government registry PDF</t>
+          <t>Official government Open Data Common registry via government CKAN mirror</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>https://migas.esdm.go.id/daftar-umum-pelumas</t>
+          <t>https://gdcatalognhic.nha.co.th/dataset/lubricant_data</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12626</v>
+        <v>5486</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>published product rows</t>
+          <t>normalized product identities</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2021-2025 list: 12,575 rows with NPT, 51 source placeholders; expiry lifecycle is computed and labelled as an inference</t>
+          <t>March 2024 full snapshot: 6,213 occurrences and 6,210 unique registration numbers; 727 exact holder-product-SAE-performance repeats consolidated with all evidence retained; three colliding numbers remain six separate source-conflict products; lifecycle inferred from published end date</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_historical_registry_snapshot</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Blue Angel DE-UZ 178</t>
+          <t>Indonesia NPT lubricant registry</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Germany / certified products</t>
+          <t>Indonesia / registered products</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product registry with XLSX export</t>
+          <t>Official public-government registry PDF</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>https://www.blauer-engel.de/de/produktwelt/schmierstoffe-und-hydraulikfluessigkeiten</t>
+          <t>https://migas.esdm.go.id/daftar-umum-pelumas</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>148</v>
+        <v>12626</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>normalized certified products</t>
+          <t>published product rows</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>149 export rows and product cards; one exact duplicate identity merged; 159 category occurrences across seven official lubricant categories; contact and marketing fields excluded</t>
+          <t>2021-2025 list: 12,575 rows with NPT, 51 source placeholders; expiry lifecycle is computed and labelled as an inference</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1293,26 +1293,26 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Korea Eco-Label EL611</t>
+          <t>Blue Angel DE-UZ 178</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Republic of Korea / certified products</t>
+          <t>Germany / certified products</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Official open-government ecolabel CSV</t>
+          <t>Official ecolabel product registry with XLSX export</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>https://www.data.go.kr/data/15043624/fileData.do</t>
+          <t>https://www.blauer-engel.de/de/produktwelt/schmierstoffe-und-hydraulikfluessigkeiten</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>240,695 file rows observed versus 99,602 in portal metadata; exact EL611 filter yields 21 lubricant rows and 20 product identities; unrestricted use; business and location identifiers excluded</t>
+          <t>149 export rows and product cards; one exact duplicate identity merged; 159 category occurrences across seven official lubricant categories; contact and marketing fields excluded</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1333,7 +1333,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Korea Eco-Label EL509</t>
+          <t>Korea Eco-Label EL611</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1352,16 +1352,16 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>normalized certified technical fluids</t>
+          <t>normalized certified products</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Exact EL509 filter yields 11 vehicle glass washer fluid rows and nine product identities after package-model merging; unrestricted use; business and location identifiers excluded</t>
+          <t>240,695 file rows observed versus 99,602 in portal metadata; exact EL611 filter yields 21 lubricant rows and 20 product identities; unrestricted use; business and location identifiers excluded</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1373,35 +1373,35 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UAE MOIAT Product Conformity</t>
+          <t>Korea Eco-Label EL509</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates / international certified products</t>
+          <t>Republic of Korea / certified products</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Official open-government certification registry</t>
+          <t>Official open-government ecolabel CSV</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>https://moiat.gov.ae/en/open-data/product-conformity-data</t>
+          <t>https://www.data.go.kr/data/15043624/fileData.do</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>1840</v>
+        <v>9</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>normalized product/model identities</t>
+          <t>normalized certified technical fluids</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>131 listing pages; 1,236 certificates; 3,176 product-certificate occurrences; explicit package suffixes and certificate renewals merged; 111 products active at snapshot; open-data page permits unrestricted reuse</t>
+          <t>Exact EL509 filter yields 11 vehicle glass washer fluid rows and nine product identities after package-model merging; unrestricted use; business and location identifiers excluded</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1413,75 +1413,75 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>US EPA Safer Choice</t>
+          <t>UAE MOIAT Product Conformity</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Arab Emirates / international certified products</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official open-government bulk CSV/API</t>
+          <t>Official open-government certification registry</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://data.epa.gov/efservice/t_safer_choice_and_design_for_the_environment/CSV</t>
+          <t>https://moiat.gov.ae/en/open-data/product-conformity-data</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2</v>
+        <v>1840</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>normalized explicitly named lubricant products</t>
+          <t>normalized product/model identities</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>12 UPC/GTIN/MPN occurrences in 4,786 source rows merged to two medical-instrument lubricants; degreasers and grease-trap cleaners excluded</t>
+          <t>131 listing pages; 1,236 certificates; 3,176 product-certificate occurrences; explicit package suffixes and certificate renewals merged; 111 products active at snapshot; open-data page permits unrestricted reuse</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>KEBS S-Mark</t>
+          <t>US EPA Safer Choice</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Kenya / locally manufactured certified products</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official government product-certification directory</t>
+          <t>Official open-government bulk CSV/API</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://www.kebs.org/products-with-smarks/</t>
+          <t>https://data.epa.gov/efservice/t_safer_choice_and_design_for_the_environment/CSV</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>750</v>
+        <v>2</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid products</t>
+          <t>normalized explicitly named lubricant products</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
+          <t>12 UPC/GTIN/MPN occurrences in 4,786 source rows merged to two medical-instrument lubricants; degreasers and grease-trap cleaners excluded</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1493,12 +1493,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>UNBS certified products</t>
+          <t>KEBS S-Mark</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Uganda / locally manufactured certified products</t>
+          <t>Kenya / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1508,20 +1508,20 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://cims.unbs.go.ug/api/website/</t>
+          <t>https://www.kebs.org/products-with-smarks/</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>46</v>
+        <v>750</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and brake-fluid products</t>
+          <t>normalized lubricant and technical-fluid products</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
+          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1533,12 +1533,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TBS certified companies</t>
+          <t>UNBS certified products</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Tanzania / locally manufactured certified products</t>
+          <t>Uganda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1548,20 +1548,20 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.tbs.go.tz/index.php/companies</t>
+          <t>https://cims.unbs.go.ug/api/website/</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>183</v>
+        <v>46</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant, coolant and brake-fluid products</t>
+          <t>normalized lubricant and brake-fluid products</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
+          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1573,35 +1573,35 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SON MANCAP Chemical Sector</t>
+          <t>TBS certified companies</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Nigeria / locally manufactured certified products</t>
+          <t>Tanzania / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official mandatory product-certification PDF</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
+          <t>https://www.tbs.go.tz/index.php/companies</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>608</v>
+        <v>183</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
+          <t>normalized lubricant, coolant and brake-fluid products</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
+          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1613,35 +1613,35 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>RSB S-Mark</t>
+          <t>SON MANCAP Chemical Sector</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Rwanda / locally manufactured certified products</t>
+          <t>Nigeria / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official government product-certification directory</t>
+          <t>Official mandatory product-certification PDF</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
+          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>9</v>
+        <v>608</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>normalized currently valid lubricant products</t>
+          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
+          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,161 +1653,161 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BIS product-certification licences</t>
+          <t>RSB S-Mark</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>India / certified manufacturers</t>
+          <t>Rwanda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official interactive government certification directory</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
+          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>normalized currently valid lubricant products</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
+          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>official_feed_or_written_access_required</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BPCL MAK Lubricants</t>
+          <t>BIS product-certification licences</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>India / international markets</t>
+          <t>India / certified manufacturers</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official interactive government certification directory</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>publicly stated minimum grades</t>
-        </is>
-      </c>
+          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
+          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>official_feed_or_written_access_required</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>BPCL MAK Lubricants</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>India / international markets</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>124</v>
+        <v>400</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>publicly stated minimum grades</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1826,7 +1826,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -1835,59 +1835,59 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1897,25 +1897,25 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1927,7 +1927,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1937,16 +1937,16 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1977,25 +1977,25 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2007,7 +2007,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2022,20 +2022,20 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2047,35 +2047,35 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2087,22 +2087,22 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
@@ -2110,12 +2110,12 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2127,47 +2127,47 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2177,31 +2177,37 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2211,71 +2217,71 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2285,64 +2291,58 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2364,11 +2364,11 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2404,11 +2404,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2484,11 +2484,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2524,11 +2524,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2604,11 +2604,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2644,11 +2644,11 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2657,12 +2657,12 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2697,12 +2697,12 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2737,12 +2737,12 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2764,11 +2764,11 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2844,11 +2844,11 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2884,11 +2884,11 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>182</v>
+        <v>756</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>649</v>
+        <v>182</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
+          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2964,11 +2964,11 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>506</v>
+        <v>649</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3004,11 +3004,11 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>640</v>
+        <v>506</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>641 embedded rows; one series excluded; informational factual fields only</t>
+          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>599</v>
+        <v>640</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
+          <t>641 embedded rows; one series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3084,11 +3084,11 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>484</v>
+        <v>599</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
+          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -3124,11 +3124,11 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>691</v>
+        <v>484</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
+          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>952</v>
+        <v>691</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
+          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -3204,11 +3204,11 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>966</v>
+        <v>952</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
+          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3234,21 +3234,21 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>1464</v>
+        <v>966</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3257,12 +3257,12 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -3274,21 +3274,21 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Republic of Korea</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>221</v>
+        <v>1464</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3297,12 +3297,12 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
+          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Republic of Korea</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -3324,11 +3324,11 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>965</v>
+        <v>221</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -3364,11 +3364,11 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>5</v>
+        <v>965</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
+          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3404,11 +3404,11 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>496</v>
+        <v>5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
+          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -3444,11 +3444,11 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>842</v>
+        <v>496</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
+          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3484,11 +3484,11 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>966</v>
+        <v>842</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -3524,20 +3524,20 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>1</v>
+        <v>966</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade row</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>One embedded concrete product card; informational factual fields only</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3564,20 +3564,20 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>975</v>
+        <v>1</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows</t>
+          <t>normalized product-grade row</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>One embedded concrete product card; informational factual fields only</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -3604,77 +3604,77 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>591</v>
+        <v>975</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>85</v>
+        <v>591</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -3684,173 +3684,173 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.zabs.org.zm/certification</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>product-certification holder records</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="n"/>
-      <c r="F80" s="2" t="n"/>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>certification records</t>
+        </is>
+      </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
         </is>
       </c>
       <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>active references</t>
-        </is>
-      </c>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -3862,81 +3862,87 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="n"/>
-      <c r="F85" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -3946,54 +3952,54 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="n"/>
-      <c r="F87" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -4005,75 +4011,75 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E88" s="2" t="n"/>
       <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E89" s="2" t="n"/>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4088,26 +4094,26 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E90" s="2" t="n"/>
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4122,14 +4128,14 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E91" s="2" t="n"/>
       <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -4141,7 +4147,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4156,14 +4162,14 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E92" s="2" t="n"/>
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -4175,7 +4181,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4190,7 +4196,7 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E93" s="2" t="n"/>
@@ -4209,7 +4215,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4219,12 +4225,12 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E94" s="2" t="n"/>
@@ -4243,7 +4249,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -4258,14 +4264,14 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E95" s="2" t="n"/>
       <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -4277,7 +4283,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4287,12 +4293,12 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E96" s="2" t="n"/>
@@ -4311,7 +4317,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -4326,14 +4332,14 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E97" s="2" t="n"/>
       <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -4345,79 +4351,113 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E98" s="2" t="n"/>
       <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="n"/>
+      <c r="F99" s="2" t="n"/>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B99" s="2" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C99" s="2" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D99" s="2" t="inlineStr">
+      <c r="D100" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E99" s="2" t="n">
+      <c r="E100" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F99" s="2" t="inlineStr">
+      <c r="F100" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G99" s="2" t="inlineStr">
+      <c r="G100" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H99" s="2" t="inlineStr">
+      <c r="H100" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H99"/>
+  <autoFilter ref="A1:H100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add official Ceypetco lubricant catalog
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -2127,35 +2127,35 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Ceypetco lubricants</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official state-owned supplier catalog + TDS</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>normalized product-grade/color rows</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2167,47 +2167,47 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2217,31 +2217,37 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2251,71 +2257,71 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2325,64 +2331,58 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2404,11 +2404,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2484,11 +2484,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2524,11 +2524,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2604,11 +2604,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2644,11 +2644,11 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2697,12 +2697,12 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2737,12 +2737,12 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2764,11 +2764,11 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2844,11 +2844,11 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2884,11 +2884,11 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>182</v>
+        <v>756</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2964,11 +2964,11 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>649</v>
+        <v>182</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
+          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3004,11 +3004,11 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>506</v>
+        <v>649</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>640</v>
+        <v>506</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>641 embedded rows; one series excluded; informational factual fields only</t>
+          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3084,11 +3084,11 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>599</v>
+        <v>640</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
+          <t>641 embedded rows; one series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -3124,11 +3124,11 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>484</v>
+        <v>599</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
+          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>691</v>
+        <v>484</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
+          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -3204,11 +3204,11 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>952</v>
+        <v>691</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
+          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3244,11 +3244,11 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>966</v>
+        <v>952</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
+          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3274,21 +3274,21 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>1464</v>
+        <v>966</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3297,12 +3297,12 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -3314,21 +3314,21 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Republic of Korea</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>221</v>
+        <v>1464</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3337,12 +3337,12 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
+          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Republic of Korea</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -3364,11 +3364,11 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>965</v>
+        <v>221</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3404,11 +3404,11 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>5</v>
+        <v>965</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
+          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -3444,11 +3444,11 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>496</v>
+        <v>5</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
+          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3484,11 +3484,11 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>842</v>
+        <v>496</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
+          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -3524,11 +3524,11 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>966</v>
+        <v>842</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3564,20 +3564,20 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>1</v>
+        <v>966</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade row</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>One embedded concrete product card; informational factual fields only</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -3604,20 +3604,20 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>975</v>
+        <v>1</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows</t>
+          <t>normalized product-grade row</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>One embedded concrete product card; informational factual fields only</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -3644,77 +3644,77 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>591</v>
+        <v>975</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>85</v>
+        <v>591</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3724,173 +3724,173 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.zabs.org.zm/certification</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>product-certification holder records</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="n"/>
-      <c r="F81" s="2" t="n"/>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>certification records</t>
+        </is>
+      </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
         </is>
       </c>
       <c r="E82" s="2" t="n"/>
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>active references</t>
-        </is>
-      </c>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>419</v>
+        <v>19000</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
@@ -3902,81 +3902,87 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="n"/>
-      <c r="F86" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -3986,54 +3992,54 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="n"/>
-      <c r="F88" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -4045,75 +4051,75 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E89" s="2" t="n"/>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E90" s="2" t="n"/>
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4128,26 +4134,26 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E91" s="2" t="n"/>
       <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4162,14 +4168,14 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E92" s="2" t="n"/>
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -4181,7 +4187,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4196,14 +4202,14 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E93" s="2" t="n"/>
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -4215,7 +4221,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4230,7 +4236,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E94" s="2" t="n"/>
@@ -4249,7 +4255,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -4259,12 +4265,12 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E95" s="2" t="n"/>
@@ -4283,7 +4289,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4298,14 +4304,14 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E96" s="2" t="n"/>
       <c r="F96" s="2" t="n"/>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -4317,7 +4323,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -4327,12 +4333,12 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E97" s="2" t="n"/>
@@ -4351,7 +4357,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4366,14 +4372,14 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E98" s="2" t="n"/>
       <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -4385,79 +4391,113 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E99" s="2" t="n"/>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="n"/>
+      <c r="F100" s="2" t="n"/>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B100" s="2" t="inlineStr">
+      <c r="B101" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
+      <c r="C101" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="D101" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E100" s="2" t="n">
+      <c r="E101" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F100" s="2" t="inlineStr">
+      <c r="F101" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G100" s="2" t="inlineStr">
+      <c r="G101" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H100" s="2" t="inlineStr">
+      <c r="H101" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H100"/>
+  <autoFilter ref="A1:H101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Record Wolf catalog rights and stabilize AIChilon hashing
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -3897,161 +3897,167 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Wolf Lubricants</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global / 27 locale variants</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official daily product sitemap and product cards</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://docs.wolfoil.com/en-us</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>419</v>
+        <v>391</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>unique branded product identities</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Exactly 391 IDs with suffix -01 observed 2026-07-21; terms prohibit substantial database reuse for any purpose</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Champion Lubricants</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global / 27 locale variants</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official daily product sitemap and product cards</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.championlubes.com/en-us/products</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>447</v>
+        <v>431</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>unique branded product identities</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>Exactly 431 IDs with suffix -02 observed 2026-07-21; same Wolf Oil Corporation database-reuse restriction</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="n"/>
-      <c r="F87" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>170</v>
+        <v>447</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>normalized lubricant and technical-fluid master products</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4061,65 +4067,71 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E89" s="2" t="n"/>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4134,14 +4146,14 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E91" s="2" t="n"/>
       <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -4153,29 +4165,29 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E92" s="2" t="n"/>
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -4187,7 +4199,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4202,26 +4214,26 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E93" s="2" t="n"/>
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4236,14 +4248,14 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E94" s="2" t="n"/>
       <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -4255,7 +4267,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -4270,14 +4282,14 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E95" s="2" t="n"/>
       <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -4289,7 +4301,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4299,12 +4311,12 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E96" s="2" t="n"/>
@@ -4323,7 +4335,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -4333,19 +4345,19 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E97" s="2" t="n"/>
       <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -4357,7 +4369,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4367,19 +4379,19 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E98" s="2" t="n"/>
       <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -4391,7 +4403,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -4401,19 +4413,19 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E99" s="2" t="n"/>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -4425,79 +4437,147 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E100" s="2" t="n"/>
       <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="n"/>
+      <c r="F101" s="2" t="n"/>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="n"/>
+      <c r="F102" s="2" t="n"/>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B101" s="2" t="inlineStr">
+      <c r="B103" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr">
+      <c r="C103" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D101" s="2" t="inlineStr">
+      <c r="D103" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E101" s="2" t="n">
+      <c r="E103" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F101" s="2" t="inlineStr">
+      <c r="F103" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G101" s="2" t="inlineStr">
+      <c r="G103" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H101" s="2" t="inlineStr">
+      <c r="H103" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H101"/>
+  <autoFilter ref="A1:H103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Integrate EAEU lubricant conformity evidence
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -563,7 +563,7 @@
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="68" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="57" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1453,75 +1453,75 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>US EPA Safer Choice</t>
+          <t>EAEU conformity-document register</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>EAEU member states / imported and domestic products</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official open-government bulk CSV/API</t>
+          <t>Official open-government OData/REST conformity register</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://data.epa.gov/efservice/t_safer_choice_and_design_for_the_environment/CSV</t>
+          <t>https://tech.eaeunion.org/tech/registers/35-1</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>2</v>
+        <v>38444</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>normalized explicitly named lubricant products</t>
+          <t>normalized manufacturer/holder + reported designation + family identities</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>12 UPC/GTIN/MPN occurrences in 4,786 source rows merged to two medical-instrument lubricants; degreasers and grease-trap cleaners excluded</t>
+          <t>81,076 unique documents across 17 exact ten-digit TN VED code slices; 51,768 candidate occurrences; 13,324 repeat certificate occurrences merged; 2,943 explicit trademarks and 35,501 clearly flagged manufacturer/holder fallbacks; register evidence is not current-market proof</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified_conservative_product_evidence</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>KEBS S-Mark</t>
+          <t>US EPA Safer Choice</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Kenya / locally manufactured certified products</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official government product-certification directory</t>
+          <t>Official open-government bulk CSV/API</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://www.kebs.org/products-with-smarks/</t>
+          <t>https://data.epa.gov/efservice/t_safer_choice_and_design_for_the_environment/CSV</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>750</v>
+        <v>2</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid products</t>
+          <t>normalized explicitly named lubricant products</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
+          <t>12 UPC/GTIN/MPN occurrences in 4,786 source rows merged to two medical-instrument lubricants; degreasers and grease-trap cleaners excluded</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1533,12 +1533,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>UNBS certified products</t>
+          <t>KEBS S-Mark</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Uganda / locally manufactured certified products</t>
+          <t>Kenya / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1548,20 +1548,20 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://cims.unbs.go.ug/api/website/</t>
+          <t>https://www.kebs.org/products-with-smarks/</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>46</v>
+        <v>750</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and brake-fluid products</t>
+          <t>normalized lubricant and technical-fluid products</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
+          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1573,12 +1573,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TBS certified companies</t>
+          <t>UNBS certified products</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Tanzania / locally manufactured certified products</t>
+          <t>Uganda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1588,20 +1588,20 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.tbs.go.tz/index.php/companies</t>
+          <t>https://cims.unbs.go.ug/api/website/</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>183</v>
+        <v>46</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant, coolant and brake-fluid products</t>
+          <t>normalized lubricant and brake-fluid products</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
+          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1613,35 +1613,35 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SON MANCAP Chemical Sector</t>
+          <t>TBS certified companies</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Nigeria / locally manufactured certified products</t>
+          <t>Tanzania / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Official mandatory product-certification PDF</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
+          <t>https://www.tbs.go.tz/index.php/companies</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>608</v>
+        <v>183</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
+          <t>normalized lubricant, coolant and brake-fluid products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
+          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,35 +1653,35 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>RSB S-Mark</t>
+          <t>SON MANCAP Chemical Sector</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Rwanda / locally manufactured certified products</t>
+          <t>Nigeria / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official government product-certification directory</t>
+          <t>Official mandatory product-certification PDF</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
+          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>9</v>
+        <v>608</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>normalized currently valid lubricant products</t>
+          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
+          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1693,161 +1693,161 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BIS product-certification licences</t>
+          <t>RSB S-Mark</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>India / certified manufacturers</t>
+          <t>Rwanda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official interactive government certification directory</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
+          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>normalized currently valid lubricant products</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
+          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>official_feed_or_written_access_required</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BPCL MAK Lubricants</t>
+          <t>BIS product-certification licences</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>India / international markets</t>
+          <t>India / certified manufacturers</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official interactive government certification directory</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>publicly stated minimum grades</t>
-        </is>
-      </c>
+          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
+          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>official_feed_or_written_access_required</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>BPCL MAK Lubricants</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>India / international markets</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>124</v>
+        <v>400</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>publicly stated minimum grades</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -1875,59 +1875,59 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1937,25 +1937,25 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1977,16 +1977,16 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2007,7 +2007,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2017,25 +2017,25 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2047,7 +2047,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2062,20 +2062,20 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2087,35 +2087,35 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2127,35 +2127,35 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Ceypetco lubricants</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official state-owned supplier catalog + TDS</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade/color rows</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2167,35 +2167,35 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Ceypetco lubricants</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official state-owned supplier catalog + TDS</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>normalized product-grade/color rows</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2207,47 +2207,47 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2257,31 +2257,37 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2291,71 +2297,71 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2365,64 +2371,58 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2484,11 +2484,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2524,11 +2524,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2604,11 +2604,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2644,11 +2644,11 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2737,12 +2737,12 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2764,11 +2764,11 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -2817,12 +2817,12 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2844,11 +2844,11 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2884,11 +2884,11 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2964,11 +2964,11 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>182</v>
+        <v>756</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3004,11 +3004,11 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>649</v>
+        <v>182</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
+          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>506</v>
+        <v>649</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3084,11 +3084,11 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>640</v>
+        <v>506</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>641 embedded rows; one series excluded; informational factual fields only</t>
+          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -3124,11 +3124,11 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>599</v>
+        <v>640</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
+          <t>641 embedded rows; one series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>484</v>
+        <v>599</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
+          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -3204,11 +3204,11 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>691</v>
+        <v>484</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
+          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3244,11 +3244,11 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>952</v>
+        <v>691</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
+          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -3284,11 +3284,11 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>966</v>
+        <v>952</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
+          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3314,21 +3314,21 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>1464</v>
+        <v>966</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3337,12 +3337,12 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -3354,21 +3354,21 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Republic of Korea</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>221</v>
+        <v>1464</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3377,12 +3377,12 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
+          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Republic of Korea</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3404,11 +3404,11 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>965</v>
+        <v>221</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -3444,11 +3444,11 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>5</v>
+        <v>965</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
+          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3484,11 +3484,11 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>496</v>
+        <v>5</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
+          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -3524,11 +3524,11 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>842</v>
+        <v>496</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
+          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3564,11 +3564,11 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>966</v>
+        <v>842</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -3604,20 +3604,20 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>1</v>
+        <v>966</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade row</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>One embedded concrete product card; informational factual fields only</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -3644,20 +3644,20 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>975</v>
+        <v>1</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows</t>
+          <t>normalized product-grade row</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>One embedded concrete product card; informational factual fields only</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -3684,77 +3684,77 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>591</v>
+        <v>975</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>85</v>
+        <v>591</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -3764,180 +3764,180 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.zabs.org.zm/certification</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>product-certification holder records</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="n"/>
-      <c r="F82" s="2" t="n"/>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>certification records</t>
+        </is>
+      </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
         </is>
       </c>
       <c r="E83" s="2" t="n"/>
       <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>active references</t>
-        </is>
-      </c>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Wolf Lubricants</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Global / 27 locale variants</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Official daily product sitemap and product cards</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://docs.wolfoil.com/en-us</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>391</v>
+        <v>19000</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>unique branded product identities</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Exactly 391 IDs with suffix -01 observed 2026-07-21; terms prohibit substantial database reuse for any purpose</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Champion Lubricants</t>
+          <t>Wolf Lubricants</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -3952,11 +3952,11 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://www.championlubes.com/en-us/products</t>
+          <t>https://docs.wolfoil.com/en-us</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>431</v>
+        <v>391</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Exactly 431 IDs with suffix -02 observed 2026-07-21; same Wolf Oil Corporation database-reuse restriction</t>
+          <t>Exactly 391 IDs with suffix -01 observed 2026-07-21; terms prohibit substantial database reuse for any purpose</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -3977,40 +3977,40 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Champion Lubricants</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global / 27 locale variants</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official daily product sitemap and product cards</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.championlubes.com/en-us/products</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>419</v>
+        <v>431</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>unique branded product identities</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Exactly 431 IDs with suffix -02 observed 2026-07-21; same Wolf Oil Corporation database-reuse restriction</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
@@ -4022,81 +4022,87 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="n"/>
-      <c r="F89" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -4106,54 +4112,54 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="n"/>
-      <c r="F91" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -4165,75 +4171,75 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E92" s="2" t="n"/>
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E93" s="2" t="n"/>
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4248,26 +4254,26 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E94" s="2" t="n"/>
       <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -4282,14 +4288,14 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E95" s="2" t="n"/>
       <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -4301,7 +4307,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4316,14 +4322,14 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E96" s="2" t="n"/>
       <c r="F96" s="2" t="n"/>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -4335,7 +4341,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -4350,7 +4356,7 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E97" s="2" t="n"/>
@@ -4369,7 +4375,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4379,12 +4385,12 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E98" s="2" t="n"/>
@@ -4403,7 +4409,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -4418,14 +4424,14 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E99" s="2" t="n"/>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -4437,7 +4443,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4447,12 +4453,12 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E100" s="2" t="n"/>
@@ -4471,7 +4477,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -4486,14 +4492,14 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E101" s="2" t="n"/>
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -4505,79 +4511,113 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E102" s="2" t="n"/>
       <c r="F102" s="2" t="n"/>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="n"/>
+      <c r="F103" s="2" t="n"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B103" s="2" t="inlineStr">
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D103" s="2" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E103" s="2" t="n">
+      <c r="E104" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F103" s="2" t="inlineStr">
+      <c r="F104" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G103" s="2" t="inlineStr">
+      <c r="G104" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H103" s="2" t="inlineStr">
+      <c r="H104" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H103"/>
+  <autoFilter ref="A1:H104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Integrate Philippine ecolabel engine oil evidence
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -1413,155 +1413,155 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>UAE MOIAT Product Conformity</t>
+          <t>Green Choice Philippines GCP 2008032</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates / international certified products</t>
+          <t>Philippines / historical certification</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Official open-government certification registry</t>
+          <t>National ecolabel public licence checker</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>https://moiat.gov.ae/en/open-data/product-conformity-data</t>
+          <t>https://pcepsdi.org.ph/check-gcp-seal/</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1840</v>
+        <v>3</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>normalized product/model identities</t>
+          <t>expired named engine-oil licences</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>131 listing pages; 1,236 certificates; 3,176 product-certificate occurrences; explicit package suffixes and certificate renewals merged; 111 products active at snapshot; open-data page permits unrestricted reuse</t>
+          <t>All three exact automotive-engine-oil rows occur only in the official Expired table; source typo SW-40 retained and flagged, not corrected by guess</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_historical_only</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>EAEU conformity-document register</t>
+          <t>UAE MOIAT Product Conformity</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>EAEU member states / imported and domestic products</t>
+          <t>United Arab Emirates / international certified products</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Official open-government OData/REST conformity register</t>
+          <t>Official open-government certification registry</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>https://tech.eaeunion.org/tech/registers/35-1</t>
+          <t>https://moiat.gov.ae/en/open-data/product-conformity-data</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>38444</v>
+        <v>1840</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>normalized manufacturer/holder + reported designation + family identities</t>
+          <t>normalized product/model identities</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>81,076 unique documents across 17 exact ten-digit TN VED code slices; 51,768 candidate occurrences; 13,324 repeat certificate occurrences merged; 2,943 explicit trademarks and 35,501 clearly flagged manufacturer/holder fallbacks; register evidence is not current-market proof</t>
+          <t>131 listing pages; 1,236 certificates; 3,176 product-certificate occurrences; explicit package suffixes and certificate renewals merged; 111 products active at snapshot; open-data page permits unrestricted reuse</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_product_evidence</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>US EPA Safer Choice</t>
+          <t>EAEU conformity-document register</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>EAEU member states / imported and domestic products</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Official open-government bulk CSV/API</t>
+          <t>Official open-government OData/REST conformity register</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>https://data.epa.gov/efservice/t_safer_choice_and_design_for_the_environment/CSV</t>
+          <t>https://tech.eaeunion.org/tech/registers/35-1</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>2</v>
+        <v>38444</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>normalized explicitly named lubricant products</t>
+          <t>normalized manufacturer/holder + reported designation + family identities</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>12 UPC/GTIN/MPN occurrences in 4,786 source rows merged to two medical-instrument lubricants; degreasers and grease-trap cleaners excluded</t>
+          <t>81,076 unique documents across 17 exact ten-digit TN VED code slices; 51,768 candidate occurrences; 13,324 repeat certificate occurrences merged; 2,943 explicit trademarks and 35,501 clearly flagged manufacturer/holder fallbacks; register evidence is not current-market proof</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified_conservative_product_evidence</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>KEBS S-Mark</t>
+          <t>US EPA Safer Choice</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Kenya / locally manufactured certified products</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Official government product-certification directory</t>
+          <t>Official open-government bulk CSV/API</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>https://www.kebs.org/products-with-smarks/</t>
+          <t>https://data.epa.gov/efservice/t_safer_choice_and_design_for_the_environment/CSV</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>750</v>
+        <v>2</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid products</t>
+          <t>normalized explicitly named lubricant products</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
+          <t>12 UPC/GTIN/MPN occurrences in 4,786 source rows merged to two medical-instrument lubricants; degreasers and grease-trap cleaners excluded</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1573,12 +1573,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>UNBS certified products</t>
+          <t>KEBS S-Mark</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Uganda / locally manufactured certified products</t>
+          <t>Kenya / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1588,20 +1588,20 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://cims.unbs.go.ug/api/website/</t>
+          <t>https://www.kebs.org/products-with-smarks/</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>46</v>
+        <v>750</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and brake-fluid products</t>
+          <t>normalized lubricant and technical-fluid products</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
+          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1613,12 +1613,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TBS certified companies</t>
+          <t>UNBS certified products</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Tanzania / locally manufactured certified products</t>
+          <t>Uganda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1628,20 +1628,20 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://www.tbs.go.tz/index.php/companies</t>
+          <t>https://cims.unbs.go.ug/api/website/</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>183</v>
+        <v>46</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant, coolant and brake-fluid products</t>
+          <t>normalized lubricant and brake-fluid products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
+          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,35 +1653,35 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SON MANCAP Chemical Sector</t>
+          <t>TBS certified companies</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Nigeria / locally manufactured certified products</t>
+          <t>Tanzania / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Official mandatory product-certification PDF</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
+          <t>https://www.tbs.go.tz/index.php/companies</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>608</v>
+        <v>183</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
+          <t>normalized lubricant, coolant and brake-fluid products</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
+          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1693,35 +1693,35 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>RSB S-Mark</t>
+          <t>SON MANCAP Chemical Sector</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Rwanda / locally manufactured certified products</t>
+          <t>Nigeria / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official government product-certification directory</t>
+          <t>Official mandatory product-certification PDF</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
+          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>9</v>
+        <v>608</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>normalized currently valid lubricant products</t>
+          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
+          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1733,161 +1733,161 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BIS product-certification licences</t>
+          <t>RSB S-Mark</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>India / certified manufacturers</t>
+          <t>Rwanda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official interactive government certification directory</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
+          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>normalized currently valid lubricant products</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
+          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>official_feed_or_written_access_required</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BPCL MAK Lubricants</t>
+          <t>BIS product-certification licences</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>India / international markets</t>
+          <t>India / certified manufacturers</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official interactive government certification directory</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>publicly stated minimum grades</t>
-        </is>
-      </c>
+          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
+          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>official_feed_or_written_access_required</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>BPCL MAK Lubricants</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>India / international markets</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>124</v>
+        <v>400</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>publicly stated minimum grades</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1906,7 +1906,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1915,59 +1915,59 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1977,25 +1977,25 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2007,7 +2007,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2017,16 +2017,16 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2047,7 +2047,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2057,25 +2057,25 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2102,20 +2102,20 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2127,35 +2127,35 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2167,35 +2167,35 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Ceypetco lubricants</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official state-owned supplier catalog + TDS</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade/color rows</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2207,35 +2207,35 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Ceypetco lubricants</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official state-owned supplier catalog + TDS</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>normalized product-grade/color rows</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2247,47 +2247,47 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2297,31 +2297,37 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2331,71 +2337,71 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2405,64 +2411,58 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2484,11 +2484,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2524,11 +2524,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2604,11 +2604,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2644,11 +2644,11 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2764,11 +2764,11 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -2817,12 +2817,12 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2844,11 +2844,11 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -2857,12 +2857,12 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2884,11 +2884,11 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2964,11 +2964,11 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3004,11 +3004,11 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>182</v>
+        <v>756</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>649</v>
+        <v>182</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
+          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3084,11 +3084,11 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>506</v>
+        <v>649</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -3124,11 +3124,11 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>640</v>
+        <v>506</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>641 embedded rows; one series excluded; informational factual fields only</t>
+          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>599</v>
+        <v>640</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
+          <t>641 embedded rows; one series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -3204,11 +3204,11 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>484</v>
+        <v>599</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
+          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3244,11 +3244,11 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>691</v>
+        <v>484</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
+          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -3284,11 +3284,11 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>952</v>
+        <v>691</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
+          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -3324,11 +3324,11 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>966</v>
+        <v>952</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
+          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -3354,21 +3354,21 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>1464</v>
+        <v>966</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3377,12 +3377,12 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -3394,21 +3394,21 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Republic of Korea</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>221</v>
+        <v>1464</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3417,12 +3417,12 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
+          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Republic of Korea</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -3444,11 +3444,11 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>965</v>
+        <v>221</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3484,11 +3484,11 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>5</v>
+        <v>965</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
+          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -3524,11 +3524,11 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>496</v>
+        <v>5</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
+          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3564,11 +3564,11 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>842</v>
+        <v>496</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
+          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -3604,11 +3604,11 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>966</v>
+        <v>842</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -3617,7 +3617,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -3644,20 +3644,20 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>1</v>
+        <v>966</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade row</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>One embedded concrete product card; informational factual fields only</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -3684,20 +3684,20 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>975</v>
+        <v>1</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows</t>
+          <t>normalized product-grade row</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>One embedded concrete product card; informational factual fields only</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3724,77 +3724,77 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>591</v>
+        <v>975</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>85</v>
+        <v>591</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3804,510 +3804,534 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.zabs.org.zm/certification</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>product-certification holder records</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="n"/>
-      <c r="F83" s="2" t="n"/>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>certification records</t>
+        </is>
+      </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
         </is>
       </c>
       <c r="E84" s="2" t="n"/>
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>BSTI CM licence lists</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official regional certification PDF lists</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://bsti.gov.bd/site/page/fae2ce93-b2cd-49c4-af5b-d2e9733d6211/List-of-companies-licensed-from-BSTI</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>19000</v>
+        <v>9</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>generic lubricant licence-class rows</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>Twenty-one PDFs reviewed; relevant rows expose holder, licence and generic standard scope, but no marketed brand, grade or product designation</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Wolf Lubricants</t>
+          <t>Taiwan MOENV ecolabel products</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Global / 27 locale variants</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Official daily product sitemap and product cards</t>
+          <t>Official open-government API</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://docs.wolfoil.com/en-us</t>
+          <t>https://data.moenv.gov.tw/dataset/detail/GP_P_02</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>391</v>
+        <v>0</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>unique branded product identities</t>
+          <t>relevant product rows</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Exactly 391 IDs with suffix -01 observed 2026-07-21; terms prohibit substantial database reuse for any purpose</t>
+          <t>All 26,488 records reviewed; 32 apparent oil hits were digital-copying ink false positives</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Champion Lubricants</t>
+          <t>Malaysia SIRIM certified products</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Global / 27 locale variants</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Official daily product sitemap and product cards</t>
+          <t>Official certified-product directory</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://www.championlubes.com/en-us/products</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="n">
-        <v>431</v>
-      </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>unique branded product identities</t>
-        </is>
-      </c>
+          <t>https://www.malaysiancertified.com.my/</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Exactly 431 IDs with suffix -02 observed 2026-07-21; same Wolf Oil Corporation database-reuse restriction</t>
+          <t>Current product search requires member authentication; no access control bypassed</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>authorized_data_access_required</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Singapore Green Labelling Scheme</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Singapore / international licensees</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official Type I ecolabel directory</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://sgls.sec.org.sg/product-categories/</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>419</v>
+        <v>0</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>lubricant product standards</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Current 58 standards across nine top-level categories contain no lubricant, grease, coolant or automotive-fluid standard</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="n">
-        <v>447</v>
-      </c>
-      <c r="F89" s="2" t="inlineStr">
-        <is>
-          <t>normalized lubricant and technical-fluid master products</t>
-        </is>
-      </c>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="n"/>
+      <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="2" t="n"/>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>active references</t>
+        </is>
+      </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>IndianOil SERVO</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>India / 35+ export countries</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official state-owned manufacturer disclosure</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+          <t>https://iocl.com/pages/servo-lubes-and-greases-overview</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>170</v>
+        <v>1600</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>finder results</t>
+          <t>marketed grades</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Official disclosure also reports 5,200+ formulations and 1,700+ active SKUs; website terms require prior written permission for republication</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>Wolf Lubricants</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / 27 locale variants</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official daily product sitemap and product cards</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="n"/>
-      <c r="F92" s="2" t="n"/>
+          <t>https://docs.wolfoil.com/en-us</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>391</v>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>unique branded product identities</t>
+        </is>
+      </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Exactly 391 IDs with suffix -01 observed 2026-07-21; terms prohibit substantial database reuse for any purpose</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Champion Lubricants</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / 27 locale variants</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official daily product sitemap and product cards</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="n"/>
-      <c r="F93" s="2" t="n"/>
+          <t>https://www.championlubes.com/en-us/products</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>431</v>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>unique branded product identities</t>
+        </is>
+      </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Exactly 431 IDs with suffix -02 observed 2026-07-21; same Wolf Oil Corporation database-reuse restriction</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="n"/>
-      <c r="F94" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>normalized product rows</t>
+        </is>
+      </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="n"/>
-      <c r="F95" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4317,19 +4341,19 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
         </is>
       </c>
       <c r="E96" s="2" t="n"/>
       <c r="F96" s="2" t="n"/>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -4341,41 +4365,47 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="n"/>
-      <c r="F97" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -4390,48 +4420,48 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E98" s="2" t="n"/>
       <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E99" s="2" t="n"/>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -4443,7 +4473,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4453,31 +4483,31 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E100" s="2" t="n"/>
       <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -4492,14 +4522,14 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E101" s="2" t="n"/>
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -4511,7 +4541,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4526,14 +4556,14 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E102" s="2" t="n"/>
       <c r="F102" s="2" t="n"/>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -4545,79 +4575,283 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E103" s="2" t="n"/>
       <c r="F103" s="2" t="n"/>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
+          <t>ENEOS</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="n"/>
+      <c r="F104" s="2" t="n"/>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Idemitsu</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="n"/>
+      <c r="F105" s="2" t="n"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial lubricants</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Repsol</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Official lubricants</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>https://lubricants.repsol.com/en/products/</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="n"/>
+      <c r="F106" s="2" t="n"/>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Gulf Oil</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gulfoilltd.com/products</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="n"/>
+      <c r="F107" s="2" t="n"/>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial product ranges</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Sinopec Lubricant</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Global / market-specific</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Official products</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sinopeclube.com/</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="n"/>
+      <c r="F108" s="2" t="n"/>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Automotive and industrial products; multilingual source review needed</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="n"/>
+      <c r="F109" s="2" t="n"/>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B104" s="2" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E104" s="2" t="n">
+      <c r="E110" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F104" s="2" t="inlineStr">
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G104" s="2" t="inlineStr">
+      <c r="G110" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H104" s="2" t="inlineStr">
+      <c r="H110" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H104"/>
+  <autoFilter ref="A1:H110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Integrate EPA ChemExpo lubricant product evidence
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$111</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,17 +555,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H110"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="57" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="57" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1573,52 +1573,52 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>KEBS S-Mark</t>
+          <t>US EPA ChemExpo / CPDat 4.1</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Kenya / locally manufactured certified products</t>
+          <t>United States / historical and current public-source records</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Official government product-certification directory</t>
+          <t>Official government CC0 product database and public PUC API</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>https://www.kebs.org/products-with-smarks/</t>
+          <t>https://comptox.epa.gov/chemexpo/</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>750</v>
+        <v>5714</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid products</t>
+          <t>normalized lubricant and technical-fluid product identities</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
+          <t>10,019 product-ID occurrences reviewed across 18 relevant or adjacent PUCs; 7,217 retained occurrences normalized to 5,714 identities after package and repeat-record merging; lifecycle is never inferred</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified_curated_scope_historical_or_current_unverified</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>UNBS certified products</t>
+          <t>KEBS S-Mark</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Uganda / locally manufactured certified products</t>
+          <t>Kenya / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1628,20 +1628,20 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https://cims.unbs.go.ug/api/website/</t>
+          <t>https://www.kebs.org/products-with-smarks/</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>46</v>
+        <v>750</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and brake-fluid products</t>
+          <t>normalized lubricant and technical-fluid products</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
+          <t>25 search slices; 4,276 visible cards; 2,897 unique permits observed; strict scope retained 775 permits and merged 25 renewals/duplicates; factual certification fields only, standard body text excluded</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1653,12 +1653,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TBS certified companies</t>
+          <t>UNBS certified products</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Tanzania / locally manufactured certified products</t>
+          <t>Uganda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1668,20 +1668,20 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>https://www.tbs.go.tz/index.php/companies</t>
+          <t>https://cims.unbs.go.ug/api/website/</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>183</v>
+        <v>46</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant, coolant and brake-fluid products</t>
+          <t>normalized lubricant and brake-fluid products</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
+          <t>13,091 public certification rows; 47 exact-scope permit occurrences; one historical renewal merged; district/location and standards body text excluded</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1693,35 +1693,35 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>SON MANCAP Chemical Sector</t>
+          <t>TBS certified companies</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Nigeria / locally manufactured certified products</t>
+          <t>Tanzania / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Official mandatory product-certification PDF</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
+          <t>https://www.tbs.go.tz/index.php/companies</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>608</v>
+        <v>183</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
+          <t>normalized lubricant, coolant and brake-fluid products</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
+          <t>2,642 public certification rows; 70 exact-scope certificates expose 184 marketed designations; one repeated occurrence merged; locations and standards body text excluded</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1733,35 +1733,35 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>RSB S-Mark</t>
+          <t>SON MANCAP Chemical Sector</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Rwanda / locally manufactured certified products</t>
+          <t>Nigeria / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Official government product-certification directory</t>
+          <t>Official mandatory product-certification PDF</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
+          <t>https://son.gov.ng/wp-content/uploads/2026/07/CHEMICAL-PRODUCTS-SECTOR_compressed.pdf</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>9</v>
+        <v>608</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>normalized currently valid lubricant products</t>
+          <t>normalized lubricant, grease, coolant and technical-fluid products</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
+          <t>233 pages and 2,011 consecutively numbered certification rows; 286 scope certificates expose 613 marketed designations; five exact notation/repeated-row duplicates merged; addresses, state and mark artwork excluded</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1773,161 +1773,161 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BIS product-certification licences</t>
+          <t>RSB S-Mark</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>India / certified manufacturers</t>
+          <t>Rwanda / locally manufactured certified products</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Official interactive government certification directory</t>
+          <t>Official government product-certification directory</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
+          <t>https://www.rsb.gov.rw/certifications/directories/products-with-s-marks-1</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>normalized currently valid lubricant products</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
+          <t>1,843 public directory rows numbered through 1,846; exact product names and standards retain eight engine oils plus one food-grade lubricant; location and contacts excluded</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>official_feed_or_written_access_required</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BPCL MAK Lubricants</t>
+          <t>BIS product-certification licences</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>India / international markets</t>
+          <t>India / certified manufacturers</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official interactive government certification directory</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>publicly stated minimum grades</t>
-        </is>
-      </c>
+          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
+          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>official_feed_or_written_access_required</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>BPCL MAK Lubricants</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>India / international markets</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>124</v>
+        <v>400</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>publicly stated minimum grades</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1955,59 +1955,59 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2017,25 +2017,25 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2047,7 +2047,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2057,16 +2057,16 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2097,25 +2097,25 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2127,7 +2127,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2142,20 +2142,20 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2167,35 +2167,35 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2207,35 +2207,35 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Ceypetco lubricants</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official state-owned supplier catalog + TDS</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade/color rows</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2247,35 +2247,35 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Ceypetco lubricants</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official state-owned supplier catalog + TDS</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>normalized product-grade/color rows</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2287,47 +2287,47 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2337,31 +2337,37 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2371,71 +2377,71 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2445,64 +2451,58 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+          <t>https://www.epc.shell.com/?lang=eng</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2524,11 +2524,11 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>623</v>
+        <v>1007</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>1464</v>
+        <v>623</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2604,11 +2604,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>690</v>
+        <v>1464</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2644,11 +2644,11 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>1007</v>
+        <v>690</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>675</v>
+        <v>1007</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>938</v>
+        <v>675</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2764,11 +2764,11 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>705</v>
+        <v>938</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>583</v>
+        <v>705</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -2817,12 +2817,12 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2844,11 +2844,11 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>289</v>
+        <v>583</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -2857,12 +2857,12 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2884,11 +2884,11 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -2897,12 +2897,12 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2914,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>1146</v>
+        <v>278</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2964,11 +2964,11 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>314</v>
+        <v>1146</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3004,11 +3004,11 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>756</v>
+        <v>314</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>182</v>
+        <v>756</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3084,11 +3084,11 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>649</v>
+        <v>182</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
+          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -3124,11 +3124,11 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>506</v>
+        <v>649</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>640</v>
+        <v>506</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>641 embedded rows; one series excluded; informational factual fields only</t>
+          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -3204,11 +3204,11 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>599</v>
+        <v>640</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
+          <t>641 embedded rows; one series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3244,11 +3244,11 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>484</v>
+        <v>599</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
+          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -3284,11 +3284,11 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>691</v>
+        <v>484</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
+          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -3324,11 +3324,11 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>952</v>
+        <v>691</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
+          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -3364,11 +3364,11 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>966</v>
+        <v>952</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
+          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -3394,21 +3394,21 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>1464</v>
+        <v>966</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3417,12 +3417,12 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -3434,21 +3434,21 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Republic of Korea</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>221</v>
+        <v>1464</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3457,12 +3457,12 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
+          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Republic of Korea</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3484,11 +3484,11 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>965</v>
+        <v>221</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -3524,11 +3524,11 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>5</v>
+        <v>965</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
+          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3564,11 +3564,11 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>496</v>
+        <v>5</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
+          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -3604,11 +3604,11 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>842</v>
+        <v>496</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -3617,7 +3617,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
+          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -3644,11 +3644,11 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>966</v>
+        <v>842</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -3684,20 +3684,20 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>1</v>
+        <v>966</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade row</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>One embedded concrete product card; informational factual fields only</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3724,20 +3724,20 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>975</v>
+        <v>1</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows</t>
+          <t>normalized product-grade row</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>One embedded concrete product card; informational factual fields only</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -3754,7 +3754,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -3764,77 +3764,77 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>591</v>
+        <v>975</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>85</v>
+        <v>591</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -3844,94 +3844,94 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.zabs.org.zm/certification</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>product-certification holder records</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="n"/>
-      <c r="F84" s="2" t="n"/>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>certification records</t>
+        </is>
+      </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>BSTI CM licence lists</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Official regional certification PDF lists</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://bsti.gov.bd/site/page/fae2ce93-b2cd-49c4-af5b-d2e9733d6211/List-of-companies-licensed-from-BSTI</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>generic lubricant licence-class rows</t>
-        </is>
-      </c>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Twenty-one PDFs reviewed; relevant rows expose holder, licence and generic standard scope, but no marketed brand, grade or product designation</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -3943,223 +3943,223 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Taiwan MOENV ecolabel products</t>
+          <t>BSTI CM licence lists</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Official open-government API</t>
+          <t>Official regional certification PDF lists</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://data.moenv.gov.tw/dataset/detail/GP_P_02</t>
+          <t>https://bsti.gov.bd/site/page/fae2ce93-b2cd-49c4-af5b-d2e9733d6211/List-of-companies-licensed-from-BSTI</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>relevant product rows</t>
+          <t>generic lubricant licence-class rows</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>All 26,488 records reviewed; 32 apparent oil hits were digital-copying ink false positives</t>
+          <t>Twenty-one PDFs reviewed; relevant rows expose holder, licence and generic standard scope, but no marketed brand, grade or product designation</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Malaysia SIRIM certified products</t>
+          <t>Taiwan MOENV ecolabel products</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Official certified-product directory</t>
+          <t>Official open-government API</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://www.malaysiancertified.com.my/</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="n"/>
-      <c r="F87" s="2" t="n"/>
+          <t>https://data.moenv.gov.tw/dataset/detail/GP_P_02</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>relevant product rows</t>
+        </is>
+      </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Current product search requires member authentication; no access control bypassed</t>
+          <t>All 26,488 records reviewed; 32 apparent oil hits were digital-copying ink false positives</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>authorized_data_access_required</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Singapore Green Labelling Scheme</t>
+          <t>Malaysia SIRIM certified products</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Singapore / international licensees</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Official Type I ecolabel directory</t>
+          <t>Official certified-product directory</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>https://sgls.sec.org.sg/product-categories/</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>lubricant product standards</t>
-        </is>
-      </c>
+          <t>https://www.malaysiancertified.com.my/</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Current 58 standards across nine top-level categories contain no lubricant, grease, coolant or automotive-fluid standard</t>
+          <t>Current product search requires member authentication; no access control bypassed</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>authorized_data_access_required</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>Singapore Green Labelling Scheme</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Singapore / international licensees</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official Type I ecolabel directory</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="n"/>
-      <c r="F89" s="2" t="n"/>
+          <t>https://sgls.sec.org.sg/product-categories/</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>lubricant product standards</t>
+        </is>
+      </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>Current 58 standards across nine top-level categories contain no lubricant, grease, coolant or automotive-fluid standard</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>active references</t>
-        </is>
-      </c>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>IndianOil SERVO</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>India / 35+ export countries</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Official state-owned manufacturer disclosure</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>https://iocl.com/pages/servo-lubes-and-greases-overview</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>1600</v>
+        <v>19000</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>marketed grades</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Official disclosure also reports 5,200+ formulations and 1,700+ active SKUs; website terms require prior written permission for republication</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -4171,47 +4171,47 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Wolf Lubricants</t>
+          <t>IndianOil SERVO</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Global / 27 locale variants</t>
+          <t>India / 35+ export countries</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Official daily product sitemap and product cards</t>
+          <t>Official state-owned manufacturer disclosure</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>https://docs.wolfoil.com/en-us</t>
+          <t>https://iocl.com/pages/servo-lubes-and-greases-overview</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>391</v>
+        <v>1600</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>unique branded product identities</t>
+          <t>marketed grades</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Exactly 391 IDs with suffix -01 observed 2026-07-21; terms prohibit substantial database reuse for any purpose</t>
+          <t>Official disclosure also reports 5,200+ formulations and 1,700+ active SKUs; website terms require prior written permission for republication</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Champion Lubricants</t>
+          <t>Wolf Lubricants</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4226,11 +4226,11 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>https://www.championlubes.com/en-us/products</t>
+          <t>https://docs.wolfoil.com/en-us</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>431</v>
+        <v>391</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -4239,7 +4239,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Exactly 431 IDs with suffix -02 observed 2026-07-21; same Wolf Oil Corporation database-reuse restriction</t>
+          <t>Exactly 391 IDs with suffix -01 observed 2026-07-21; terms prohibit substantial database reuse for any purpose</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -4251,40 +4251,40 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>LIQUI MOLY</t>
+          <t>Champion Lubricants</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Global English / 2020 historical</t>
+          <t>Global / 27 locale variants</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Official downloadable PDF product catalog</t>
+          <t>Official daily product sitemap and product cards</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
+          <t>https://www.championlubes.com/en-us/products</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>419</v>
+        <v>431</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>normalized product rows</t>
+          <t>unique branded product identities</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
+          <t>Exactly 431 IDs with suffix -02 observed 2026-07-21; same Wolf Oil Corporation database-reuse restriction</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_historical_factual_fields_only</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
@@ -4296,81 +4296,87 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>GB English / current 2026</t>
+          <t>Global English / 2020 historical</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Official XML sitemap + public OpenAPI</t>
+          <t>Official downloadable PDF product catalog</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+          <t>https://www.liqui-moly.com/fileadmin/user_upload/Downloads/Technische_Informationen/Kataloge_und_Prospekte/EN/5603.pdf</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>normalized lubricant and technical-fluid master products</t>
+          <t>normalized product rows</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
+          <t>204-page document dated 2020-04-23; 1,482 unique part numbers; lifecycle historical/unverified; factual fields only</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_current_factual_fields_only</t>
+          <t>ingested_and_verified_historical_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Castrol</t>
+          <t>LIQUI MOLY</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>GB English / current 2026</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Official product finder</t>
+          <t>Official XML sitemap + public OpenAPI</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>https://www.castrol.com/en/global/corporate/products.html</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="n"/>
-      <c r="F96" s="2" t="n"/>
+          <t>https://www.liqui-moly.com/sitemap/www.liqui-moly.com/sitemap_gb_en.xml</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>normalized lubricant and technical-fluid master products</t>
+        </is>
+      </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial ranges; market variants must be retained</t>
+          <t>759 sitemap product URLs; 742 resolved by API; 447 in professional scope; 985 article SKUs; factual fields only; explicit 2020→2026 lifecycle audit</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>ingested_and_verified_current_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>MOLYKOTE / DuPont</t>
+          <t>Castrol</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Global / location-filtered</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -4380,54 +4386,54 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="F97" s="2" t="inlineStr">
-        <is>
-          <t>finder results</t>
-        </is>
-      </c>
+          <t>https://www.castrol.com/en/global/corporate/products.html</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="n"/>
+      <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
+          <t>Automotive and industrial ranges; market variants must be retained</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Klüber Lubrication</t>
+          <t>MOLYKOTE / DuPont</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global / location-filtered</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official product finder</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>https://www.klueber.com/global/en/products-service/products/</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="n"/>
-      <c r="F98" s="2" t="n"/>
+          <t>https://www.dupont.com/solution-finder/results.html?BU=molykote</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>finder results</t>
+        </is>
+      </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
+          <t>Terms prohibit page-scrape/copying; written permission or licensed feed required</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -4439,75 +4445,75 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Klüber Lubrication</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Maintenance and lubrication products</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
+          <t>https://www.klueber.com/global/en/products-service/products/</t>
         </is>
       </c>
       <c r="E99" s="2" t="n"/>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
+          <t>Terms explicitly prohibit data mining, robots, scraper and offline reader</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Petro-Canada Lubricants</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Maintenance and lubrication products</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.petro-canada.com/en-ca/products</t>
+          <t>https://www.skf.com/group/products/maintenance-products/lubrication-management</t>
         </is>
       </c>
       <c r="E100" s="2" t="n"/>
       <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit screen scraping without express permission</t>
+          <t>Greases, oils and lubrication-system consumables; exclude equipment</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Chevron Lubricants</t>
+          <t>Petro-Canada Lubricants</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -4522,26 +4528,26 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
+          <t>https://lubricants.petro-canada.com/en-ca/products</t>
         </is>
       </c>
       <c r="E101" s="2" t="n"/>
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Delo, Havoline and industrial products</t>
+          <t>Terms prohibit screen scraping without express permission</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Valvoline</t>
+          <t>Chevron Lubricants</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4556,14 +4562,14 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>https://www.valvolineglobal.com/en/products/</t>
+          <t>https://www.chevronlubricants.com/en_us/home/products.html</t>
         </is>
       </c>
       <c r="E102" s="2" t="n"/>
       <c r="F102" s="2" t="n"/>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Automotive oils and fluids; region-specific availability</t>
+          <t>Delo, Havoline and industrial products</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -4575,7 +4581,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>PETRONAS Lubricants</t>
+          <t>Valvoline</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -4590,14 +4596,14 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>https://global.pli-petronas.com/products</t>
+          <t>https://www.valvolineglobal.com/en/products/</t>
         </is>
       </c>
       <c r="E103" s="2" t="n"/>
       <c r="F103" s="2" t="n"/>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial lubricants</t>
+          <t>Automotive oils and fluids; region-specific availability</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
@@ -4609,7 +4615,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>ENEOS</t>
+          <t>PETRONAS Lubricants</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -4624,7 +4630,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneos-global.com/products/lubricants/</t>
+          <t>https://global.pli-petronas.com/products</t>
         </is>
       </c>
       <c r="E104" s="2" t="n"/>
@@ -4643,7 +4649,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Idemitsu</t>
+          <t>ENEOS</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -4653,12 +4659,12 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Official lubricants</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>https://www.idemitsu.com/en/business/lube/</t>
+          <t>https://www.eneos-global.com/products/lubricants/</t>
         </is>
       </c>
       <c r="E105" s="2" t="n"/>
@@ -4677,7 +4683,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Repsol</t>
+          <t>Idemitsu</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -4692,14 +4698,14 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.repsol.com/en/products/</t>
+          <t>https://www.idemitsu.com/en/business/lube/</t>
         </is>
       </c>
       <c r="E106" s="2" t="n"/>
       <c r="F106" s="2" t="n"/>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial product ranges</t>
+          <t>Automotive and industrial lubricants</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -4711,7 +4717,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Gulf Oil</t>
+          <t>Repsol</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -4721,12 +4727,12 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Official products</t>
+          <t>Official lubricants</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>https://www.gulfoilltd.com/products</t>
+          <t>https://lubricants.repsol.com/en/products/</t>
         </is>
       </c>
       <c r="E107" s="2" t="n"/>
@@ -4745,7 +4751,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Sinopec Lubricant</t>
+          <t>Gulf Oil</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -4760,14 +4766,14 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>https://www.sinopeclube.com/</t>
+          <t>https://www.gulfoilltd.com/products</t>
         </is>
       </c>
       <c r="E108" s="2" t="n"/>
       <c r="F108" s="2" t="n"/>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Automotive and industrial products; multilingual source review needed</t>
+          <t>Automotive and industrial product ranges</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -4779,79 +4785,113 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>DEUTZ DQC</t>
+          <t>Sinopec Lubricant</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Official oil and coolant release lists</t>
+          <t>Official products</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+          <t>https://www.sinopeclube.com/</t>
         </is>
       </c>
       <c r="E109" s="2" t="n"/>
       <c r="F109" s="2" t="n"/>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+          <t>Automotive and industrial products; multilingual source review needed</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>discovery</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
+          <t>DEUTZ DQC</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Global OEM approvals</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Official oil and coolant release lists</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deutz.com/germany/en/parts-service/operating-liquids/technical-information/</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="n"/>
+      <c r="F110" s="2" t="n"/>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Current issue 07/2026 located; copyright notice requires permission for transformed/commercial reuse</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>permission_or_licensed_feed_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
           <t>Detroit / Daimler Truck DFS</t>
         </is>
       </c>
-      <c r="B110" s="2" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>North America / global suppliers</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>Official approved-fluids PDF lists</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
+      <c r="D111" s="2" t="inlineStr">
         <is>
           <t>https://dtnacontent-dtna.prd.freightliner.com/content/public/dtnaportalpublic/LubricantsFuelsCoolants.html</t>
         </is>
       </c>
-      <c r="E110" s="2" t="n">
+      <c r="E111" s="2" t="n">
         <v>661</v>
       </c>
-      <c r="F110" s="2" t="inlineStr">
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>approval occurrences</t>
         </is>
       </c>
-      <c r="G110" s="2" t="inlineStr">
+      <c r="G111" s="2" t="inlineStr">
         <is>
           <t>11 current lists dated 2026-07-09; terms restrict reuse to noncommercial personal use, therefore products are not ingested</t>
         </is>
       </c>
-      <c r="H110" s="2" t="inlineStr">
+      <c r="H111" s="2" t="inlineStr">
         <is>
           <t>written_permission_required</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H110"/>
+  <autoFilter ref="A1:H111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Integrate Pakistan PSQCA engine oil licence evidence
</commit_message>
<xml_diff>
--- a/deliverables/Global_lubricants_catalog_registry.xlsx
+++ b/deliverables/Global_lubricants_catalog_registry.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_Паспорт'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_Источники'!$A$1:$H$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_Оценка_объёма'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_Схема_данных'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_Дедупликация'!$A$1:$C$9</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -1813,161 +1813,161 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BIS product-certification licences</t>
+          <t>PSQCA CM licence verification</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>India / certified manufacturers</t>
+          <t>Pakistan / certified manufacturers</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Official interactive government certification directory</t>
+          <t>Official government product-certification licence directory</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
+          <t>https://icq.psqca.com.pk/e_services/t_cmverify.aspx</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>certified engine-oil brand scopes</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
+          <t>Two exact PS 343 engine-oil filters expose 14 CM licences: one valid and 13 expired at snapshot; these are brand-level scopes, not individual SAE/API grades</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>official_feed_or_written_access_required</t>
+          <t>ingested_and_verified_conservative_brand_scope</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BPCL MAK Lubricants</t>
+          <t>BIS product-certification licences</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>India / international markets</t>
+          <t>India / certified manufacturers</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official interactive government certification directory</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>publicly stated minimum grades</t>
-        </is>
-      </c>
+          <t>https://www.manakonline.in/MANAK/ApplicationLicenceRelatedrpt</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
+          <t>Schema exposes licence, manufacturer, IS, variety and brands, but report generation is CAPTCHA-protected; no bypass attempted</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>official_feed_or_written_access_required</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Japan Eco Mark Category 110</t>
+          <t>BPCL MAK Lubricants</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Japan / certified products</t>
+          <t>India / international markets</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Official ecolabel product search</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
+          <t>https://www.bharatpetroleum.in/our-businesses/mak-lubricants/about-mak-lubricants</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>124</v>
+        <v>400</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>current certified search entries</t>
+          <t>publicly stated minimum grades</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
+          <t>Official page reports 400+ grades; terms require prior written permission for copying or republication, so no product rows imported</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>permission_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 9150</t>
+          <t>Japan Eco Mark Category 110</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>United States / international qualified sources</t>
+          <t>Japan / certified products</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database</t>
+          <t>Official ecolabel product search</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>https://qpldocs.dla.mil/search/default.aspx</t>
+          <t>https://www.ecomark.jp/search/op_item_list.php?rkw=1&amp;ruigata=1102</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>431</v>
+        <v>124</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>normalized qualified products</t>
+          <t>current certified search entries</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
+          <t>Live count observed 2026-07-21; site policy restricts republication and processed use, so only count and source link retained pending written permission</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>permission_required</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>DLA QPD FSC 6850 lubricant scope</t>
+          <t>DLA QPD FSC 9150</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Official government qualified-products database, curated professional subset</t>
+          <t>Official government qualified-products database</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>25</v>
+        <v>431</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1995,59 +1995,59 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
+          <t>56 active QPLs; 455 product occurrences; GREEN/YELLOW/RED, SAM and Stop Ship retained separately; plant-only rows and personal/contact fields excluded</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_curated_scope</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ZF TE-ML</t>
+          <t>DLA QPD FSC 6850 lubricant scope</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Global OEM approvals</t>
+          <t>United States / international qualified sources</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Official approved-lubricant ZIP/PDF registry</t>
+          <t>Official government qualified-products database, curated professional subset</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
+          <t>https://qpldocs.dla.mil/search/default.aspx</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1498</v>
+        <v>25</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>unique approval numbers</t>
+          <t>normalized qualified products</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
+          <t>Six of 24 active FSC 6850 QPLs retained because the governing title explicitly establishes oil, silicone compound, cleaning-lubricating compound or fuel-lubricity function; pure cleaners and unrelated chemicals excluded</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified</t>
+          <t>ingested_and_verified_curated_scope</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Allison TES approved fluids</t>
+          <t>ZF TE-ML</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2057,25 +2057,25 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Official approved-fluid PDF registry</t>
+          <t>Official approved-lubricant ZIP/PDF registry</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
+          <t>https://aftermarket.zf.com/lubricants/en/2026-07-01_en.zip</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>104</v>
+        <v>1498</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>approved products</t>
+          <t>unique approval numbers</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
+          <t>4,919 approval occurrences across 28 TE-ML lists dated 2026-07-01</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Driventic DIWA approved oils</t>
+          <t>Allison TES approved fluids</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2097,16 +2097,16 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Official approved-oil PDF registry</t>
+          <t>Official approved-fluid PDF registry</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
+          <t>https://allisontransmission.com/en-gb/aftermarket---channel/parts---service/allison-approved-fluids</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>226</v>
+        <v>104</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
+          <t>Six current TES lists; 119 approval-number occurrences and 117 unique approval numbers</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2127,7 +2127,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz Trucks DTFR</t>
+          <t>Driventic DIWA approved oils</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2137,25 +2137,25 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Official operating-fluids approval API</t>
+          <t>Official approved-oil PDF registry</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>https://bevo.mercedes-benz-trucks.com/</t>
+          <t>https://www.driventic.com/products/bus/diwa-automatic-transmission</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1892</v>
+        <v>226</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>unique DTFR product IDs</t>
+          <t>approved products</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
+          <t>Four currently published highest-version lists for 60,000 to 240,000 km oil-change intervals; source list dates retained</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2167,7 +2167,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz BeVo</t>
+          <t>Mercedes-Benz Trucks DTFR</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2182,20 +2182,20 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>https://operatingfluids.mercedes-benz.com/</t>
+          <t>https://bevo.mercedes-benz-trucks.com/</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1913</v>
+        <v>1892</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>normalized approved products</t>
+          <t>unique DTFR product IDs</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
+          <t>2,102 approval occurrences across 63 product sheets; historical-only approvals retain lifecycle status</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2207,35 +2207,35 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Volvo Genuine Fluids</t>
+          <t>Mercedes-Benz BeVo</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Official manufacturer product catalog</t>
+          <t>Official operating-fluids approval API</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
+          <t>https://operatingfluids.mercedes-benz.com/</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>32</v>
+        <v>1913</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>specific product-grade rows</t>
+          <t>normalized approved products</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
+          <t>2,461 approval occurrences across 92 product sheets; 158 products cross-matched to Trucks DTFR</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2247,35 +2247,35 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Ceypetco lubricants</t>
+          <t>Volvo Genuine Fluids</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Volvo CE Asia / Volvo Trucks US-CA</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Official state-owned supplier catalog + TDS</t>
+          <t>Official manufacturer product catalog</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
+          <t>https://www.volvoce.com/asia/en-as/parts/maintenance-parts/lubricants/</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade/color rows</t>
+          <t>specific product-grade rows</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
+          <t>Five official catalog pages; ungraded VDS series excluded from product count</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2287,35 +2287,35 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>MAN current service products</t>
+          <t>Ceypetco lubricants</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>MAN trucks / global English document</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Official current OEM service recommendation</t>
+          <t>Official state-owned supplier catalog + TDS</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
+          <t>https://ceypetco.gov.lk/ceypetco-lubricants/</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>named products</t>
+          <t>normalized product-grade/color rows</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
+          <t>23 official product lines and 22 current TDS files; two source-document conflicts preserved as quality flags; factual fields only</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2327,47 +2327,47 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>API EOLCS</t>
+          <t>MAN current service products</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>MAN trucks / global English document</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Official licensed engine-oil directory</t>
+          <t>Official current OEM service recommendation</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+          <t>https://public.man.eu/media/service/asp/media/en/927247.pdf</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>35174</v>
+        <v>32</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>licensed product rows</t>
+          <t>named products</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
+          <t>April 2026 edition; 33 recommendation occurrences; standards and ungraded series excluded</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>written_permission_or_official_feed_required</t>
+          <t>ingested_and_verified</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>NSF White Book</t>
+          <t>API EOLCS</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2377,31 +2377,37 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Official nonfood compounds registry</t>
+          <t>Official licensed engine-oil directory</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
+          <t>https://engineoil.api.org/Directory/EolcsProductResults?accountId=-1</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>35174</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>licensed product rows</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
+          <t>Live 2026-07-21 count: 35,174 products from 883 companies; API terms prohibit bulk copying/republication, so only aggregate evidence is retained</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>terms_and_feed_review_required</t>
+          <t>written_permission_or_official_feed_required</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>NSF White Book</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2411,178 +2417,166 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Product catalog</t>
+          <t>Official nonfood compounds registry</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>1246</v>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
+          <t>https://info.nsf.org/USDA/psnclistings.asp</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
+          <t>Food-grade lubricants and related compounds; public search available, bulk rights and feed must be confirmed</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>terms_and_feed_review_required</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>Flender T7300</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global OEM approvals</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>EPC product catalog</t>
+          <t>Official approved-lubricants pages</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>https://www.epc.shell.com/?lang=eng</t>
+          <t>https://www.flender.com/en/approvedlubricants</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>TDS/SDS by market; copying is restricted by site terms</t>
+          <t>Current approval tables are public, but Flender Terms of Use prohibit copying, reproducing or exploiting site content without written consent</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>permission_or_permitted_access_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Mobil</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Global / market-specific</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Industrial product search</t>
+          <t>Product catalog</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
+          <t>https://lubricants.catalog.totalenergies.com/corporate/en_UK</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>1246</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Terms prohibit bots; permitted feed or written permission required</t>
+          <t>Count observed 2026-07-20; GTCU 4.3 prohibits substantial database extraction/reuse</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>permission_or_licensed_feed_required</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>EPC product catalog</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="n">
-        <v>1007</v>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.epc.shell.com/?lang=eng</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
+          <t>TDS/SDS by market; copying is restricted by site terms</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_permitted_access_required</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>FUCHS</t>
+          <t>Mobil</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Global / market-specific</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Industrial product search</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="n">
-        <v>623</v>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>normalized product-grade rows</t>
-        </is>
-      </c>
+          <t>https://www.mobil.com/en/lubricants/for-businesses/industrial/lubricants/search</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
+          <t>Terms prohibit bots; permitted feed or written permission required</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_factual_fields_only</t>
+          <t>permission_or_licensed_feed_required</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2588,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2604,11 +2598,11 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/in/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>1464</v>
+        <v>1007</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2617,7 +2611,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
+          <t>1,115 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only, descriptions omitted</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2634,7 +2628,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2644,11 +2638,11 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/us/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>690</v>
+        <v>623</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2657,7 +2651,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
+          <t>686 embedded rows; 60 series excluded; 3 duplicate occurrences merged; factual fields only; exact India overlaps reconciled by name and professional family</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2674,7 +2668,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2684,11 +2678,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/de/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>1007</v>
+        <v>1464</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2697,7 +2691,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
+          <t>1,464 concrete catalog cards; no series or duplicate occurrences; factual fields only; cross-market identity reconciled by exact name and professional family</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2714,7 +2708,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2724,11 +2718,11 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>675</v>
+        <v>690</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2737,7 +2731,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
+          <t>776 embedded rows; 81 localized series/group rows excluded; 5 duplicate occurrences merged; Polish taxonomy normalized to professional families; factual fields only</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2754,7 +2748,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2764,11 +2758,11 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/it/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>938</v>
+        <v>1007</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -2777,7 +2771,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>1,174 embedded rows; 84 series and 4 equipment rows excluded; 79 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2794,7 +2788,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2804,11 +2798,11 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/se/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>705</v>
+        <v>675</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2811,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
+          <t>675 concrete cards; no series, equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2834,7 +2828,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2844,11 +2838,11 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/es/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>583</v>
+        <v>938</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -2857,12 +2851,12 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
+          <t>1,017 embedded rows; 69 series, 6 equipment rows and 1 test placeholder excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_conservative_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2868,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2884,11 +2878,11 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>289</v>
+        <v>705</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -2897,7 +2891,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
+          <t>765 embedded rows; 42 series and 1 equipment row excluded; 17 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2914,7 +2908,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2924,11 +2918,11 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/tr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>278</v>
+        <v>583</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -2937,12 +2931,12 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>632 embedded rows; 44 series and 2 equipment rows excluded; 3 duplicate occurrences merged; no general website imprint found, conservative factual-only publication</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_conservative_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2948,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2964,11 +2958,11 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ca/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>1146</v>
+        <v>289</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -2977,12 +2971,12 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
+          <t>323 embedded rows; 34 series excluded; no equipment or duplicate occurrences; factual fields only</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -2994,7 +2988,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3004,11 +2998,11 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cn/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>314</v>
+        <v>278</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3017,7 +3011,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>364 embedded rows; 50 series excluded; factual fields only</t>
+          <t>281 embedded rows; 2 series excluded; 1 duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3034,7 +3028,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3044,11 +3038,11 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cz/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>756</v>
+        <v>1146</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3057,7 +3051,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
+          <t>1,253 embedded rows; 98 series and 6 equipment rows excluded; 3 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3074,7 +3068,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3084,11 +3078,11 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/mx/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>182</v>
+        <v>314</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3097,7 +3091,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>364 embedded rows; 50 series excluded; factual fields only</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3114,7 +3108,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -3124,11 +3118,11 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/za/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>649</v>
+        <v>756</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3137,7 +3131,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
+          <t>864 embedded rows; 94 series and 6 equipment rows excluded; 8 duplicate occurrences merged; factual fields only</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3154,7 +3148,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3164,11 +3158,11 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/br/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>506</v>
+        <v>182</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3177,7 +3171,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
+          <t>213 embedded rows; 30 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3194,7 +3188,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -3204,11 +3198,11 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/no/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>640</v>
+        <v>649</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3217,7 +3211,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>641 embedded rows; one series excluded; informational factual fields only</t>
+          <t>650 embedded rows; one series excluded; no duplicate occurrences; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3234,7 +3228,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3244,11 +3238,11 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/hu/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>599</v>
+        <v>506</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3257,7 +3251,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
+          <t>544 embedded rows; 37 series excluded; one duplicate occurrence merged; informational factual fields only under official imprint</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3274,7 +3268,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -3284,11 +3278,11 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/dk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>484</v>
+        <v>640</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3297,7 +3291,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
+          <t>641 embedded rows; one series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3314,7 +3308,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -3324,11 +3318,11 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/fi/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>691</v>
+        <v>599</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3337,7 +3331,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
+          <t>639 embedded rows; 38 series excluded; two duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -3354,7 +3348,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -3364,11 +3358,11 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/pt/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>952</v>
+        <v>484</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3377,7 +3371,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
+          <t>529 embedded rows; 42 series and two equipment rows excluded; one duplicate merged</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -3394,7 +3388,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3404,11 +3398,11 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ro/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>966</v>
+        <v>691</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3417,7 +3411,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
+          <t>794 embedded rows; 91 series and one equipment row excluded; 11 duplicates merged</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3434,21 +3428,21 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/at/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>1464</v>
+        <v>952</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3457,12 +3451,12 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
+          <t>1,057 embedded rows; 94 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3468,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Republic of Korea</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -3484,11 +3478,11 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/gr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>221</v>
+        <v>966</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -3497,7 +3491,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicates merged</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3514,21 +3508,21 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Official embedded product finder</t>
+          <t>Official embedded product finder with Germany taxonomy reconciliation</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ch/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>965</v>
+        <v>1464</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -3537,12 +3531,12 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>1,453 exact Germany-name matches reconcile 203 family differences and all 234 fallback rows; 11 unique Swiss products retain source classification</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>ingested_and_verified_informational_factual_fields_only</t>
+          <t>ingested_and_verified_cross_market_taxonomy_reconciled</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3548,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Republic of Korea</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3564,11 +3558,11 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/kr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>5</v>
+        <v>221</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -3577,7 +3571,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
+          <t>249 embedded rows; 28 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -3594,7 +3588,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -3604,11 +3598,11 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ae/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>496</v>
+        <v>965</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -3617,7 +3611,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
+          <t>1,073 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -3634,7 +3628,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -3644,11 +3638,11 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ar/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>842</v>
+        <v>5</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -3657,7 +3651,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
+          <t>35 embedded rows; 30 series excluded; informational factual fields only</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -3674,7 +3668,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -3684,11 +3678,11 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/cl/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>966</v>
+        <v>496</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -3697,7 +3691,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>549 embedded rows; 49 series and four equipment rows excluded</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -3714,7 +3708,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3724,20 +3718,20 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/ua/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>1</v>
+        <v>842</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade row</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>One embedded concrete product card; informational factual fields only</t>
+          <t>918 embedded rows; 65 series, six equipment rows and one blank placeholder excluded; four duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -3754,7 +3748,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -3764,11 +3758,11 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/sk/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>975</v>
+        <v>966</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -3777,7 +3771,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
+          <t>1,074 embedded rows; 97 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -3794,7 +3788,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Belgium / Benelux</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3804,134 +3798,140 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
+          <t>https://www.fuchs.com/si/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>591</v>
+        <v>1</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>normalized product-grade rows observed</t>
+          <t>normalized product-grade row</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
+          <t>One embedded concrete product card; informational factual fields only</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>ZABS certified products</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>https://www.zabs.org.zm/certification</t>
+          <t>https://www.fuchs.com/hr/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>85</v>
+        <v>975</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>product-certification holder records</t>
+          <t>normalized product-grade rows</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
+          <t>1,082 embedded rows; 96 series and six equipment rows excluded; five duplicate occurrences merged</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>ingested_and_verified_informational_factual_fields_only</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>BOBS product certification register</t>
+          <t>FUCHS</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Belgium / Benelux</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Official government certification register</t>
+          <t>Official embedded product finder</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>https://bobstandards.bw/product-certification-register-2/</t>
+          <t>https://www.fuchs.com/be/en/products/service-links/product-finder/</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>120</v>
+        <v>591</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>certification records</t>
+          <t>normalized product-grade rows observed</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
+          <t>673 embedded rows; official imprint prohibits copying and republication except personal non-commercial downloads</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>written_permission_required</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>SABS certified clients</t>
+          <t>ZABS certified products</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Official government certification search</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabs.co.za/sabs-certified-clients</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="n"/>
-      <c r="F85" s="2" t="n"/>
+          <t>https://www.zabs.org.zm/certification</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>product-certification holder records</t>
+        </is>
+      </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
+          <t>Public register has 181 total certification records; product tabs expose 85 holder-standard records, including Mount Meru Lubricants and two Willowton Oil records, but no marketed product/SKU names</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -3943,136 +3943,136 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>BSTI CM licence lists</t>
+          <t>BOBS product certification register</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Official regional certification PDF lists</t>
+          <t>Official government certification register</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>https://bsti.gov.bd/site/page/fae2ce93-b2cd-49c4-af5b-d2e9733d6211/List-of-companies-licensed-from-BSTI</t>
+          <t>https://bobstandards.bw/product-certification-register-2/</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>9</v>
+        <v>120</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>generic lubricant licence-class rows</t>
+          <t>certification records</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Twenty-one PDFs reviewed; relevant rows expose holder, licence and generic standard scope, but no marketed brand, grade or product designation</t>
+          <t>All 120 public rows reviewed at the snapshot; no lubricant, grease, coolant or technical-fluid product scope found</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>reviewed_no_product_sku_rows</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Taiwan MOENV ecolabel products</t>
+          <t>SABS certified clients</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Official open-government API</t>
+          <t>Official government certification search</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>https://data.moenv.gov.tw/dataset/detail/GP_P_02</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>relevant product rows</t>
-        </is>
-      </c>
+          <t>https://www.sabs.co.za/sabs-certified-clients</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>All 26,488 records reviewed; 32 apparent oil hits were digital-copying ink false positives</t>
+          <t>Searchable system and product-client register exposes company, permit, specification and scope; lubricant-related queries returned organizations and adjacent products, not marketed lubricant SKU names</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>reviewed_zero_relevant_product_rows</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Malaysia SIRIM certified products</t>
+          <t>BSTI CM licence lists</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Official certified-product directory</t>
+          <t>Official regional certification PDF lists</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>https://www.malaysiancertified.com.my/</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="n"/>
-      <c r="F88" s="2" t="n"/>
+          <t>https://bsti.gov.bd/site/page/fae2ce93-b2cd-49c4-af5b-d2e9733d6211/List-of-companies-licensed-from-BSTI</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>generic lubricant licence-class rows</t>
+        </is>
+      </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Current product search requires member authentication; no access control bypassed</t>
+          <t>Twenty-one PDFs reviewed; relevant rows expose holder, licence and generic standard scope, but no marketed brand, grade or product designation</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>authorized_data_access_required</t>
+          <t>reviewed_no_product_sku_rows</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Singapore Green Labelling Scheme</t>
+          <t>Taiwan MOENV ecolabel products</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Singapore / international licensees</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Official Type I ecolabel directory</t>
+          <t>Official open-government API</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>https://sgls.sec.org.sg/product-categories/</t>
+          <t>https://data.moenv.gov.tw/dataset/detail/GP_P_02</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
@@ -4080,12 +4080,12 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>lubricant product standards</t>
+          <t>relevant product rows</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Current 58 standards across nine top-level categories contain no lubricant, grease, coolant or automotive-fluid standard</t>
+          <t>All 26,488 records reviewed; 32 apparent oil hits were digital-copying ink false positives</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -4097,355 +4097,355 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>GSA certified clients</t>
+          <t>Malaysia SIRIM certified products</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Official government system-certification search</t>
+          <t>Official certified-product directory</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+          <t>https://www.malaysiancertified.com.my/</t>
         </is>
       </c>
       <c r="E90" s="2" t="n"/>
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
+          <t>Current product search requires member authentication; no access control bypassed</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>reviewed_not_a_product_catalog</t>
+          <t>authorized_data_access_required</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Motul</t>
+          <t>Singapore Green Labelling Scheme</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Singapore / international licensees</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Corporate disclosure</t>
+          <t>Official Type I ecolabel directory</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
+          <t>https://sgls.sec.org.sg/product-categories/</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>19000</v>
+        <v>0</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>active references</t>
+          <t>lubricant product standards</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
+          <t>Current 58 standards across nine top-level categories contain no lubricant, grease, coolant or automotive-fluid standard</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>reviewed_zero_relevant_product_rows</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>IndianOil SERVO</t>
+          <t>GSA certified clients</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>India / 35+ export countries</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Official state-owned manufacturer disclosure</t>
+          <t>Official government system-certification search</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>https://iocl.com/pages/servo-lubes-and-greases-overview</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="n">
-        <v>1600</v>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>marketed grades</t>
-        </is>
-      </c>
+          <t>https://www.gsa.gov.gh/CertificationSearch.php</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Official disclosure also reports 5,200+ formulations and 1,700+ active SKUs; website terms require prior written permission for republication</t>
+          <t>Current public search is for system-certified clients and does not expose a bulk product/SKU directory</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>count_evidence_only_permission_required</t>
+          <t>reviewed_not_a_product_catalog</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Wolf Lubricants</t>
+          <t>Motul</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Global / 27 locale variants</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Official daily product sitemap and product cards</t>
+          <t>Corporate disclosure</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>https://docs.wolfoil.com/en-us</t>
+          <t>https://cms.motul.com/images/DPEF_2024_english_e9953e284f.pdf</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>391</v>
+        <v>19000</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>unique branded product identities</t>
+          <t>active references</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Exactly 391 IDs with suffix -01 observed 2026-07-21; terms prohibit substantial database reuse for any purpose</t>
+          <t>Also reports more than 400 formulations; references are not normalized products; catalog extraction requires written permission</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>written_permission_required</t>
+          <t>count_evidence_only_permission_required</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Champion Lubricants</t>
+          <t>IndianOil SERVO</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Global / 27 locale variants</t>
+          <t>India / 35+ export countries</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Official daily product sitemap and product cards</t>
+          <t>Official state-owned manufacturer disclosure</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>https://www.championlubes.com/en-us/products</t>
+          <t>https://iocl.com/pages/servo-lubes-and-greases-overview</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>431</v>
+        <v>1600</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>unique branded product identities</